<commit_message>
feat(spark): SSV Phase A — subtract VSR depositor-liability from prime_agent_revenue (#114)
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4811785.126404739</v>
+        <v>2975150.085934307</v>
       </c>
     </row>
     <row r="5">
@@ -501,7 +501,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>4811785.126404739</v>
+        <v>2975150.085934307</v>
       </c>
     </row>
     <row r="8">
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>4811785.126404739</v>
+        <v>2975150.085934307</v>
       </c>
     </row>
     <row r="22">
@@ -625,7 +625,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-3680960.981141949</v>
+        <v>-5517596.021612381</v>
       </c>
     </row>
     <row r="25">
@@ -660,7 +660,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-05T08:15:13+00:00</t>
+          <t>2026-06-05T12:56:39+00:00</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S54"/>
+  <dimension ref="A1:S58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -857,13 +857,13 @@
         <v>1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>1786482.833459468</v>
+        <v>1454465.949905966</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>1786482.833459468</v>
+        <v>1454465.949905966</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-1786482.833459468</v>
+        <v>-1454465.949905966</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -922,13 +922,13 @@
         <v>1</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>1658929.40805144</v>
+        <v>1350618.260706183</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>1658929.40805144</v>
+        <v>1350618.260706183</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>-1658929.408051447</v>
+        <v>-1350618.26070619</v>
       </c>
       <c r="Q3" s="6" t="n">
         <v>0</v>
@@ -987,13 +987,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>1162563.717392334</v>
+        <v>946501.8694127946</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>1162563.717392334</v>
+        <v>946501.8694127946</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>-195998.1193593341</v>
+        <v>20063.72862020546</v>
       </c>
       <c r="Q4" s="6" t="n">
         <v>0</v>
@@ -1052,13 +1052,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>864046.4912132345</v>
+        <v>703463.9108016299</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>864046.4912132345</v>
+        <v>703463.9108016299</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>33345.58832489169</v>
+        <v>193928.1687364963</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>82530624.22670487</v>
@@ -1075,12 +1075,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S14</t>
+          <t>S56</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Maple syrupUSDC (ERC-4626)</t>
+          <t>Spark Savings V2 — spUSDC vault</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1090,44 +1090,44 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>300001048.426836</v>
+        <v>215278739.036717</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>100000608.9318128</v>
+        <v>207131500.431691</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-200000439.4950232</v>
+        <v>-8147238.605026</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>850905.4612414049</v>
+        <v>-635707.8750376763</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>850905.4612414049</v>
+        <v>-635707.8750376763</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>189794075.6409658</v>
+        <v>215278739.036717</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>657555.3856097412</v>
+        <v>607233.2434632853</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>657555.3856097412</v>
+        <v>607233.2434632853</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>193350.0756316637</v>
+        <v>-1242941.118500961</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>0</v>
@@ -1140,59 +1140,59 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S5</t>
+          <t>S60</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Spark PYUSD (SparkLend spToken)</t>
+          <t>Spark Savings V2 — spUSDC vault (Avalanche-C, CREATE2 same address)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>avalanche_c</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>144386807.117522</v>
+        <v>190414182.348414</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>99995755.66040599</v>
+        <v>95656876.179346</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>-44391051.457116</v>
+        <v>-94757306.16906799</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>238689.828336</v>
+        <v>-651003.1837891456</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>238689.828336</v>
+        <v>-651003.1837891456</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>142947138.0437977</v>
+        <v>190414182.348414</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>495250.7614411016</v>
+        <v>537098.1921680442</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>495250.7614411016</v>
+        <v>537098.1921680442</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-256560.9331051016</v>
+        <v>-1188101.37595719</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>0</v>
@@ -1205,12 +1205,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S25</t>
+          <t>S14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Spark.fi PYUSD Reserve Curve (PYUSD/USDS)</t>
+          <t>Maple syrupUSDC (ERC-4626)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1220,44 +1220,44 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>100000415.9451873</v>
+        <v>300001048.426836</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>100000425.5500491</v>
+        <v>100000608.9318128</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>9.604861756901659</v>
+        <v>-200000439.4950232</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>7431.658583213117</v>
+        <v>850905.4612414049</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>7431.658583213117</v>
+        <v>850905.4612414049</v>
       </c>
       <c r="K8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>100000176.5240995</v>
+        <v>189794075.6409658</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>346457.8881784314</v>
+        <v>535349.067247757</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>346457.8881784314</v>
+        <v>535349.067247757</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-339026.2295952183</v>
+        <v>315556.3939936479</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>0</v>
@@ -1270,12 +1270,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S57</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Spark USDS (SparkLend spToken)</t>
+          <t>Spark Savings V2 — spUSDT vault</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1285,331 +1285,331 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>177429260.508884</v>
+        <v>153856441.430568</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>556639355.9139084</v>
+        <v>120038508.359851</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>379210095.4050245</v>
+        <v>-33817933.070717</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>458278.510553758</v>
+        <v>-549209.6068296075</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>458278.510553758</v>
+        <v>-549209.6068296075</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>94458108.0135076</v>
+        <v>153856441.430568</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>327256.9885494479</v>
+        <v>433980.3659927064</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>327256.9885494479</v>
+        <v>433980.3659927064</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>131021.5220043101</v>
+        <v>-983189.972822314</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>95188953.04035926</v>
+        <v>0</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>(avg excl. lending_idle)</t>
-        </is>
-      </c>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S43</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Arbitrum — POL)</t>
+          <t>Spark PYUSD (SparkLend spToken)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>178950.6498946011</v>
+        <v>144386807.117522</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>196264917.5470026</v>
+        <v>99995755.66040599</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>196085966.8971079</v>
+        <v>-44391051.457116</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0</v>
+        <v>238689.828336</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0</v>
+        <v>238689.828336</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>82302337.13128559</v>
+        <v>142947138.0437977</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>285142.4358014278</v>
+        <v>403208.6710770108</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>264203.5578583014</v>
+        <v>403208.6710770108</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>-285142.4358014278</v>
+        <v>-164518.8427410108</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>20938.87794312634</v>
+        <v>0</v>
       </c>
       <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S37</t>
+          <t>S25</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Base — POL)</t>
+          <t>Spark.fi PYUSD Reserve Curve (PYUSD/USDS)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>74829605.8002511</v>
+        <v>100000415.9451873</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>75079284.39269957</v>
+        <v>100000425.5500491</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>249678.5924484764</v>
+        <v>9.604861756901659</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0</v>
+        <v>7431.658583213117</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0</v>
+        <v>7431.658583213117</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>74829605.8002511</v>
+        <v>100000176.5240995</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>259252.6143444519</v>
+        <v>282068.8740994219</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>240214.90488203</v>
+        <v>282068.8740994219</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>-259252.6143444519</v>
+        <v>-274637.2155162088</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>19037.70946242194</v>
+        <v>0</v>
       </c>
       <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S34</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Spark USDC Vault (Morpho, Base)</t>
+          <t>Spark USDS (SparkLend spToken)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>167771852.1309772</v>
+        <v>177429260.508884</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>61.15121926789406</v>
+        <v>556639355.9139084</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-167771790.9797579</v>
+        <v>379210095.4050245</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>218121.4647922712</v>
+        <v>458278.510553758</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>218121.4647922712</v>
+        <v>458278.510553758</v>
       </c>
       <c r="K12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>48672080.32484906</v>
+        <v>94458108.0135076</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>168627.9639569869</v>
+        <v>266436.45144477</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>168627.9639569869</v>
+        <v>266436.45144477</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>49493.50083528426</v>
+        <v>191842.059108988</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>0</v>
+        <v>95188953.04035926</v>
       </c>
       <c r="R12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>(avg excl. lending_idle)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S43</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Spark USDC (SparkLend spToken)</t>
+          <t>Savings USDS / sUSDS proxy (Arbitrum — POL)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>43177397.521021</v>
+        <v>178950.6498946011</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>43659321.092129</v>
+        <v>196264917.5470026</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>481923.571108</v>
+        <v>196085966.8971079</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>145492.432133</v>
+        <v>0</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>145492.432133</v>
+        <v>0</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>43188250.13840729</v>
+        <v>82302337.13128559</v>
       </c>
       <c r="M13" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>149628.8352397903</v>
+        <v>232148.8659050326</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>149628.8352397903</v>
+        <v>211209.9879619063</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>-4136.403106790296</v>
+        <v>-232148.8659050326</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>0</v>
+        <v>20938.87794312634</v>
       </c>
       <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S47</t>
+          <t>S37</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Optimism — POL)</t>
+          <t>Savings USDS / sUSDS proxy (Base — POL)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1618,13 +1618,13 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>970178.1267029551</v>
+        <v>74829605.8002511</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>101106912.9085265</v>
+        <v>75079284.39269957</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>100136734.7818235</v>
+        <v>249678.5924484764</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>0</v>
@@ -1639,42 +1639,42 @@
         <v>0</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>42907533.96338371</v>
+        <v>74829605.8002511</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>148656.273624834</v>
+        <v>211070.6539832326</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>137739.990469148</v>
+        <v>192032.9445208107</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>-148656.273624834</v>
+        <v>-211070.6539832326</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>10916.28315568595</v>
+        <v>19037.70946242194</v>
       </c>
       <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S18</t>
+          <t>S34</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Arkis Spark Prime USDC 1 (ERC-4626)</t>
+          <t>Spark USDC Vault (Morpho, Base)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1683,40 +1683,40 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>15024030.59441916</v>
+        <v>167771852.1309772</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>15106645.23632516</v>
+        <v>61.15121926789406</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>82614.64190600339</v>
+        <v>-167771790.9797579</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>82614.64190600339</v>
+        <v>218121.4647922712</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>82614.64190600339</v>
+        <v>218121.4647922712</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>15024030.59441916</v>
+        <v>48672080.32484906</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>52051.84723265141</v>
+        <v>137288.5466256973</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>52051.84723265141</v>
+        <v>137288.5466256973</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>30562.79467335199</v>
+        <v>80832.91816657386</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>0</v>
@@ -1729,138 +1729,142 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SPREAD</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>30bps sUSDS spread (Curve LP + PSM3) — Sky Revenue reduction</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+          <t>Spark USDC (SparkLend spToken)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="E16" s="6" t="n">
-        <v>0</v>
+        <v>43177397.521021</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>0</v>
+        <v>43659321.092129</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0</v>
+        <v>481923.571108</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0</v>
+        <v>145492.432133</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>0</v>
+        <v>145492.432133</v>
       </c>
       <c r="K16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>0</v>
+        <v>43188250.13840729</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0</v>
+        <v>121820.3958662906</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>-39145.45144251771</v>
+        <v>121820.3958662906</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>0</v>
+        <v>23672.03626670938</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>39145.45144251771</v>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>sky-revenue reduction (no CoF; computed outside venue loop)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S54</t>
+          <t>S47</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aave Avalanche USDC (aAvaUSDC)</t>
+          <t>Savings USDS / sUSDS proxy (Optimism — POL)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>optimism</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>10000438.058711</v>
+        <v>970178.1267029551</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>10000965.036792</v>
+        <v>101106912.9085265</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>526.978081</v>
+        <v>100136734.7818235</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>31596.950878</v>
+        <v>0</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>31596.950878</v>
+        <v>0</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>9999435.801524</v>
+        <v>42907533.96338371</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>34643.7729531098</v>
+        <v>121028.5843097249</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>34643.7729531098</v>
+        <v>110112.3011540389</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>-3046.822075109799</v>
+        <v>-121028.5843097249</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>0</v>
+        <v>10916.28315568595</v>
       </c>
       <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S24</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
+          <t>Arkis Spark Prime USDC 1 (ERC-4626)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1870,178 +1874,170 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>50000864.48440416</v>
+        <v>15024030.59441916</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>49999911.74966041</v>
+        <v>15106645.23632516</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-952.7347437553233</v>
+        <v>82614.64190600339</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>82614.64190600339</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0</v>
+        <v>82614.64190600339</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>0</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>49999946.74995758</v>
+        <v>15024030.59441916</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>0</v>
+        <v>42378.03913457882</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>42378.03913457882</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>0</v>
+        <v>40236.60277142459</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>49999946.74995758</v>
+        <v>0</v>
       </c>
       <c r="R18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>SDE (fixed)</t>
-        </is>
-      </c>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>SPREAD</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Spark Blue Chip USDC Vault (Morpho)</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>30bps sUSDS spread (Curve LP + PSM3) — Sky Revenue reduction</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" s="6" t="n">
-        <v>10124757.36060807</v>
+        <v>0</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>976334.4376037563</v>
+        <v>0</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>-9148422.923004312</v>
+        <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>22913.63278708834</v>
+        <v>0</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>22913.63278708834</v>
+        <v>0</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>6870535.567559426</v>
+        <v>0</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>23803.47041505258</v>
+        <v>0</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>23803.47041505258</v>
+        <v>-39145.45144251771</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>-889.8376279642375</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" t="inlineStr"/>
+        <v>39145.45144251771</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>sky-revenue reduction (no CoF; computed outside venue loop)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S53</t>
+          <t>S54</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>USDC raw (Unichain — ALM idle)</t>
+          <t>Aave Avalanche USDC (aAvaUSDC)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>avalanche_c</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>5000000</v>
+        <v>10000438.058711</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>5000000</v>
+        <v>10000965.036792</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0</v>
+        <v>526.978081</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>8e-12</v>
+        <v>31596.950878</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>8e-12</v>
+        <v>31596.950878</v>
       </c>
       <c r="K20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>5000180.50613029</v>
+        <v>9999435.801524</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>17323.48920651527</v>
+        <v>28205.24619259639</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>17323.48920651527</v>
+        <v>28205.24619259639</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>-17323.48920651527</v>
+        <v>3391.704685403611</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -2054,124 +2050,128 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>S45</t>
+          <t>S24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>USDC raw (Arbitrum — ALM idle)</t>
+          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>5000000</v>
+        <v>50000864.48440416</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>4994817.315553</v>
+        <v>49999911.74966041</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>-5182.684447</v>
+        <v>-952.7347437553233</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>4.83813e-09</v>
+        <v>27497.03310050249</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4.83813e-09</v>
+        <v>0</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0</v>
+        <v>27497.03310050249</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>4993920.215864256</v>
+        <v>49999946.74995758</v>
       </c>
       <c r="M21" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>17301.79997535245</v>
+        <v>0</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17301.79997535245</v>
+        <v>27497.03310050249</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-17301.79997534761</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>0</v>
+        <v>49999946.74995758</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>SDE (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S49</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>USDC raw (Optimism — ALM idle)</t>
+          <t>Spark Blue Chip USDC Vault (Morpho)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>5000000</v>
+        <v>10124757.36060807</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>5000000</v>
+        <v>976334.4376037563</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0</v>
+        <v>-9148422.923004312</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1.658e-09</v>
+        <v>22913.63278708834</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>1.658e-09</v>
+        <v>22913.63278708834</v>
       </c>
       <c r="K22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>4980707.317678578</v>
+        <v>6870535.567559426</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>17256.02292813871</v>
+        <v>19379.60811033649</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>17256.02292813871</v>
+        <v>19379.60811033649</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>-17256.02292813705</v>
+        <v>3534.024676751853</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2184,17 +2184,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S39</t>
+          <t>S53</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>USDC raw (Base — ALM idle)</t>
+          <t>USDC raw (Unichain — ALM idle)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>unichain</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2203,40 +2203,40 @@
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>4732058.263226</v>
+        <v>5000000</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>4979093.435761</v>
+        <v>5000000</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>247035.172535</v>
+        <v>0</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>-9.9179e-08</v>
+        <v>8e-12</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>-9.9179e-08</v>
+        <v>8e-12</v>
       </c>
       <c r="K23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>4948516.885305397</v>
+        <v>5000180.50613029</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17144.49683281351</v>
+        <v>14103.92795974866</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>17144.49683281351</v>
+        <v>14103.92795974866</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>-17144.49683291269</v>
+        <v>-14103.92795974865</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
@@ -2249,82 +2249,82 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S51</t>
+          <t>S45</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Unichain — POL)</t>
+          <t>USDC raw (Arbitrum — ALM idle)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>970178.1267029551</v>
+        <v>5000000</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>973415.2506528809</v>
+        <v>4994817.315553</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>3237.123949925721</v>
+        <v>-5182.684447</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0</v>
+        <v>4.83813e-09</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0</v>
+        <v>4.83813e-09</v>
       </c>
       <c r="K24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>970178.1267029551</v>
+        <v>4993920.215864256</v>
       </c>
       <c r="M24" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>3361.252715923034</v>
+        <v>14086.26966065105</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>3114.425686628358</v>
+        <v>14086.26966065105</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>-3361.252715923034</v>
+        <v>-14086.26966064621</v>
       </c>
       <c r="Q24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>246.8270292946761</v>
+        <v>0</v>
       </c>
       <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>S55</t>
+          <t>S49</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>USDC raw (Avalanche-C — ALM idle)</t>
+          <t>USDC raw (Optimism — ALM idle)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>optimism</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2333,40 +2333,40 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-5.6e-10</v>
+        <v>1.658e-09</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>-5.6e-10</v>
+        <v>1.658e-09</v>
       </c>
       <c r="K25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>1629.366092641322</v>
+        <v>4980707.317678578</v>
       </c>
       <c r="M25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>5.645057390373821</v>
+        <v>14049.00025329229</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>5.645057390373821</v>
+        <v>14049.00025329229</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>-5.645057390933821</v>
+        <v>-14049.00025329063</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -2379,59 +2379,59 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S39</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Spark DAI Vault (Morpho)</t>
+          <t>USDC raw (Base — ALM idle)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>286.4890802084861</v>
+        <v>4732058.263226</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>332.9212943539781</v>
+        <v>4979093.435761</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>46.432214145492</v>
+        <v>247035.172535</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>2.378383224018197</v>
+        <v>-9.9179e-08</v>
       </c>
       <c r="I26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>2.378383224018197</v>
+        <v>-9.9179e-08</v>
       </c>
       <c r="K26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>314.5978487958594</v>
+        <v>4948516.885305397</v>
       </c>
       <c r="M26" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>1.089947139173536</v>
+        <v>13958.2012234117</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>1.089947139173536</v>
+        <v>13958.2012234117</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>1.28843608484466</v>
+        <v>-13958.20122351087</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>0</v>
@@ -2444,17 +2444,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>S36</t>
+          <t>S51</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS, Base)</t>
+          <t>Savings USDS / sUSDS proxy (Unichain — POL)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>unichain</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2463,13 +2463,13 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>283.8972488542868</v>
+        <v>970178.1267029551</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>283.8972488542868</v>
+        <v>973415.2506528809</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0</v>
+        <v>3237.123949925721</v>
       </c>
       <c r="H27" s="6" t="n">
         <v>0</v>
@@ -2484,37 +2484,37 @@
         <v>0</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>283.8972488542868</v>
+        <v>970178.1267029551</v>
       </c>
       <c r="M27" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>0.9835826767167647</v>
+        <v>2736.56568805195</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>0.9835826767167647</v>
+        <v>2489.738658757273</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>-0.9835826767167647</v>
+        <v>-2736.56568805195</v>
       </c>
       <c r="Q27" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>0</v>
+        <v>246.8270292946761</v>
       </c>
       <c r="S27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>S16</t>
+          <t>S59</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ethena Staked USDe (sUSDe)</t>
+          <t>Spark Savings V2 — spPYUSD vault</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2524,44 +2524,44 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>98.2186939487863</v>
+        <v>21463.341472</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>98.60727406618892</v>
+        <v>285387.136685</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>0.3885801174026364</v>
+        <v>263923.795213</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.3885801174026364</v>
+        <v>-714.374814002612</v>
       </c>
       <c r="I28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0.3885801174026364</v>
+        <v>-714.374814002612</v>
       </c>
       <c r="K28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>98.2186939487863</v>
+        <v>21463.341472</v>
       </c>
       <c r="M28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>0.340285812164936</v>
+        <v>60.5412987642022</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>0.340285812164936</v>
+        <v>60.5412987642022</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.04829430523770046</v>
+        <v>-774.9161127668142</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>0</v>
@@ -2574,17 +2574,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>S27</t>
+          <t>S55</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>USDT raw (ALM idle — $442M as of 2026-04)</t>
+          <t>USDC raw (Avalanche-C — ALM idle)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>avalanche_c</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2602,31 +2602,31 @@
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>9.05e-10</v>
+        <v>-5.6e-10</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>9.05e-10</v>
+        <v>-5.6e-10</v>
       </c>
       <c r="K29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>63.38209825078258</v>
+        <v>1629.366092641322</v>
       </c>
       <c r="M29" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>0.2195918914502308</v>
+        <v>4.595926479553287</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>0.2195918914502308</v>
+        <v>4.595926479553287</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>-0.2195918905452308</v>
+        <v>-4.595926480113287</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -2639,12 +2639,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Spark USDS Vault (Morpho)</t>
+          <t>Spark DAI Vault (Morpho)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2658,40 +2658,40 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>21.8939178481358</v>
+        <v>286.4890802084861</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>21.90604334087989</v>
+        <v>332.9212943539781</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>0.01212549274409835</v>
+        <v>46.432214145492</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.000970031078014375</v>
+        <v>2.378383224018197</v>
       </c>
       <c r="I30" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.000970031078014375</v>
+        <v>2.378383224018197</v>
       </c>
       <c r="K30" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>21.89559878438257</v>
+        <v>314.5978487958594</v>
       </c>
       <c r="M30" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>0.07585889524316237</v>
+        <v>0.8873810435980858</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>0.07585889524316237</v>
+        <v>0.8873810435980858</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>-0.07488886416514801</v>
+        <v>1.491002180420111</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>0</v>
@@ -2704,59 +2704,59 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>S23</t>
+          <t>S36</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Anchorage tri-party loan escrow (USDC pass-through, ~$0 balance)</t>
+          <t>Fluid Savings USDS (fsUSDS, Base)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1.111098</v>
+        <v>283.8972488542868</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>1.210584</v>
+        <v>283.8972488542868</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>0.099486</v>
+        <v>0</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.099486</v>
+        <v>0</v>
       </c>
       <c r="I31" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.099486</v>
+        <v>0</v>
       </c>
       <c r="K31" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>1.111098</v>
+        <v>283.8972488542868</v>
       </c>
       <c r="M31" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>0.003849479871133108</v>
+        <v>0.8007843598651403</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>0.003849479871133108</v>
+        <v>0.8007843598651403</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>0.09563652012886689</v>
+        <v>-0.8007843598651403</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>0</v>
@@ -2769,12 +2769,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>S8</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Aave Ethereum USDC (aToken)</t>
+          <t>Ethena Staked USDe (sUSDe)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2784,44 +2784,44 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.057177</v>
+        <v>98.2186939487863</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>0.057354</v>
+        <v>98.60727406618892</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>0.000177</v>
+        <v>0.3885801174026364</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.000177</v>
+        <v>0.3885801174026364</v>
       </c>
       <c r="I32" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.000177</v>
+        <v>0.3885801174026364</v>
       </c>
       <c r="K32" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>0.057177</v>
+        <v>98.2186939487863</v>
       </c>
       <c r="M32" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>0.000198093877040349</v>
+        <v>0.2770438751272927</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0.000198093877040349</v>
+        <v>0.2770438751272927</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>-2.109387704034901e-05</v>
+        <v>0.1115362422753438</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -2834,59 +2834,59 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>S41</t>
+          <t>S27</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Aave Arbitrum USDCn (aArbUSDCn)</t>
+          <t>USDT raw (ALM idle — $442M as of 2026-04)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0.006294</v>
+        <v>0</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>0.00631</v>
+        <v>0</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>1.6e-05</v>
+        <v>0</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>1.6e-05</v>
+        <v>9.05e-10</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>1.6e-05</v>
+        <v>9.05e-10</v>
       </c>
       <c r="K33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L33" s="6" t="n">
-        <v>0.006294</v>
+        <v>63.38209825078258</v>
       </c>
       <c r="M33" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>2.180602098906827e-05</v>
+        <v>0.1787808553252768</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>2.180602098906827e-05</v>
+        <v>0.1787808553252768</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>-5.806020989068273e-06</v>
+        <v>-0.1787808544202768</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -2899,12 +2899,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Aave Ethereum USDS (aToken)</t>
+          <t>Spark USDS Vault (Morpho)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2914,44 +2914,44 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>0.005735356645015577</v>
+        <v>21.8939178481358</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>0.005739369858543872</v>
+        <v>21.90604334087989</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>4.013213528295e-06</v>
+        <v>0.01212549274409835</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>4.013213528295e-06</v>
+        <v>0.000970031078014375</v>
       </c>
       <c r="I34" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>4.013213528295e-06</v>
+        <v>0.000970031078014375</v>
       </c>
       <c r="K34" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>0.005735356645015577</v>
+        <v>21.89559878438257</v>
       </c>
       <c r="M34" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>1.987056043549442e-05</v>
+        <v>0.0617605599461623</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>1.987056043549442e-05</v>
+        <v>0.0617605599461623</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-1.585734690719942e-05</v>
+        <v>-0.06079052886814793</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>0</v>
@@ -2964,59 +2964,59 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>S35</t>
+          <t>S23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Aave Base USDC (aBasUSDC)</t>
+          <t>Anchorage tri-party loan escrow (USDC pass-through, ~$0 balance)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>0.001682</v>
+        <v>1.111098</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>0.001688</v>
+        <v>1.210584</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>6e-06</v>
+        <v>0.099486</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>6e-06</v>
+        <v>0.099486</v>
       </c>
       <c r="I35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>6e-06</v>
+        <v>0.099486</v>
       </c>
       <c r="K35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L35" s="6" t="n">
-        <v>0.001682</v>
+        <v>1.111098</v>
       </c>
       <c r="M35" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>5.827411392375729e-06</v>
+        <v>0.00313405608637691</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>5.827411392375729e-06</v>
+        <v>0.00313405608637691</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>1.725886076242714e-07</v>
+        <v>0.09635194391362309</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -3029,12 +3029,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>S17</t>
+          <t>S8</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS)</t>
+          <t>Aave Ethereum USDC (aToken)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3044,44 +3044,44 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>0.001240144670509943</v>
+        <v>0.057177</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>0.001240144670509943</v>
+        <v>0.057354</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>0</v>
+        <v>0.000177</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0</v>
+        <v>0.000177</v>
       </c>
       <c r="I36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0</v>
+        <v>0.000177</v>
       </c>
       <c r="K36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>0.001240144670509943</v>
+        <v>0.057177</v>
       </c>
       <c r="M36" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>4.29657145132205e-06</v>
+        <v>0.0001612782354488736</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>4.29657145132205e-06</v>
+        <v>0.0001612782354488736</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>-4.29657145132205e-06</v>
+        <v>1.572176455112641e-05</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>0</v>
@@ -3094,17 +3094,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S41</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Aave Ethereum Lido USDS (aToken)</t>
+          <t>Aave Arbitrum USDCn (aArbUSDCn)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3113,40 +3113,40 @@
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>0.000281702874169182</v>
+        <v>0.006294</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>0.000518423030497757</v>
+        <v>0.00631</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>0.000236720156328575</v>
+        <v>1.6e-05</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>4.89352007537e-07</v>
+        <v>1.6e-05</v>
       </c>
       <c r="I37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>4.89352007537e-07</v>
+        <v>1.6e-05</v>
       </c>
       <c r="K37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>0.0002893232226956671</v>
+        <v>0.006294</v>
       </c>
       <c r="M37" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.002381357916522e-06</v>
+        <v>1.775338359681708e-05</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>1.002381357916522e-06</v>
+        <v>1.775338359681708e-05</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>-5.130293503795222e-07</v>
+        <v>-1.753383596817084e-06</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>0</v>
@@ -3159,12 +3159,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>S7</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>USDe raw (ALM idle)</t>
+          <t>Aave Ethereum USDS (aToken)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3174,44 +3174,44 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>7.4896275897803e-05</v>
+        <v>0.005735356645015577</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>7.4896275897803e-05</v>
+        <v>0.005739369858543872</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>0</v>
+        <v>4.013213528295e-06</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0</v>
+        <v>4.013213528295e-06</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>0</v>
+        <v>4.013213528295e-06</v>
       </c>
       <c r="K38" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>7.4896275897803e-05</v>
+        <v>0.005735356645015577</v>
       </c>
       <c r="M38" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.594835977487354e-07</v>
+        <v>1.61776273567708e-05</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>2.594835977487354e-07</v>
+        <v>1.61776273567708e-05</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>-2.594835977487354e-07</v>
+        <v>-1.21644138284758e-05</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>0</v>
@@ -3224,59 +3224,59 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S29</t>
+          <t>S35</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DAI raw (ALM idle)</t>
+          <t>Aave Base USDC (aBasUSDC)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>0</v>
+        <v>0.001682</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>0</v>
+        <v>0.001688</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>0</v>
+        <v>6e-06</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>-1.08687469e-07</v>
+        <v>6e-06</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>-1.08687469e-07</v>
+        <v>6e-06</v>
       </c>
       <c r="K39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>7.243125283870968e-08</v>
+        <v>0.001682</v>
       </c>
       <c r="M39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>2.509433459906918e-10</v>
+        <v>4.744390087360396e-06</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>2.509433459906918e-10</v>
+        <v>4.744390087360396e-06</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>-1.089384123459907e-07</v>
+        <v>1.255609912639604e-06</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -3289,12 +3289,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>S17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Aave Ethereum USDT (aToken)</t>
+          <t>Fluid Savings USDS (fsUSDS)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3304,14 +3304,14 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>0</v>
+        <v>0.001240144670509943</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>0</v>
+        <v>0.001240144670509943</v>
       </c>
       <c r="G40" s="6" t="n">
         <v>0</v>
@@ -3329,19 +3329,19 @@
         <v>0</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>0</v>
+        <v>0.001240144670509943</v>
       </c>
       <c r="M40" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>0</v>
+        <v>3.498055934399643e-06</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>0</v>
+        <v>3.498055934399643e-06</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>0</v>
+        <v>-3.498055934399643e-06</v>
       </c>
       <c r="Q40" s="6" t="n">
         <v>0</v>
@@ -3354,12 +3354,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Spark Blue Chip USDT Vault (Morpho V2)</t>
+          <t>Aave Ethereum Lido USDS (aToken)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3369,44 +3369,44 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>0</v>
+        <v>0.000281702874169182</v>
       </c>
       <c r="F41" s="6" t="n">
-        <v>0</v>
+        <v>0.000518423030497757</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>0</v>
+        <v>0.000236720156328575</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0</v>
+        <v>4.89352007537e-07</v>
       </c>
       <c r="I41" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J41" s="6" t="n">
-        <v>0</v>
+        <v>4.89352007537e-07</v>
       </c>
       <c r="K41" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L41" s="6" t="n">
-        <v>0</v>
+        <v>0.0002893232226956671</v>
       </c>
       <c r="M41" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>0</v>
+        <v>8.160893161715145e-07</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>0</v>
+        <v>8.160893161715145e-07</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>0</v>
+        <v>-3.267373086345146e-07</v>
       </c>
       <c r="Q41" s="6" t="n">
         <v>0</v>
@@ -3419,12 +3419,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S15</t>
+          <t>S30</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Maple syrupUSDT (ERC-4626)</t>
+          <t>USDe raw (ALM idle)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3434,14 +3434,14 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>0</v>
+        <v>7.4896275897803e-05</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>0</v>
+        <v>7.4896275897803e-05</v>
       </c>
       <c r="G42" s="6" t="n">
         <v>0</v>
@@ -3459,19 +3459,19 @@
         <v>0</v>
       </c>
       <c r="L42" s="6" t="n">
-        <v>0</v>
+        <v>7.4896275897803e-05</v>
       </c>
       <c r="M42" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N42" s="6" t="n">
-        <v>0</v>
+        <v>2.112587092447954e-07</v>
       </c>
       <c r="O42" s="6" t="n">
-        <v>0</v>
+        <v>2.112587092447954e-07</v>
       </c>
       <c r="P42" s="6" t="n">
-        <v>0</v>
+        <v>-2.112587092447954e-07</v>
       </c>
       <c r="Q42" s="6" t="n">
         <v>0</v>
@@ -3484,12 +3484,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S19</t>
+          <t>S29</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
+          <t>DAI raw (ALM idle)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
@@ -3512,31 +3512,31 @@
         <v>0</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>0</v>
+        <v>-1.08687469e-07</v>
       </c>
       <c r="I43" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>0</v>
+        <v>-1.08687469e-07</v>
       </c>
       <c r="K43" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L43" s="6" t="n">
-        <v>0</v>
+        <v>7.243125283870968e-08</v>
       </c>
       <c r="M43" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N43" s="6" t="n">
-        <v>0</v>
+        <v>2.043056587295296e-10</v>
       </c>
       <c r="O43" s="6" t="n">
-        <v>0</v>
+        <v>2.043056587295296e-10</v>
       </c>
       <c r="P43" s="6" t="n">
-        <v>0</v>
+        <v>-1.088917746587295e-07</v>
       </c>
       <c r="Q43" s="6" t="n">
         <v>0</v>
@@ -3549,12 +3549,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S20</t>
+          <t>S9</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Janus Henderson Anemoy Treasury Fund (JTRSY)</t>
+          <t>Aave Ethereum USDT (aToken)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
@@ -3614,12 +3614,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S21</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Superstate Short Duration US Government Securities Fund (USTB)</t>
+          <t>Spark Blue Chip USDT Vault (Morpho V2)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
@@ -3657,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N45" s="6" t="n">
         <v>0</v>
@@ -3674,21 +3674,17 @@
       <c r="R45" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>SDE (fixed)</t>
-        </is>
-      </c>
+      <c r="S45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S22</t>
+          <t>S15</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Superstate Crypto Carry Fund (USCC)</t>
+          <t>Maple syrupUSDT (ERC-4626)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3698,7 +3694,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
@@ -3748,12 +3744,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>S26</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>USDC raw (ALM idle)</t>
+          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3763,7 +3759,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
@@ -3776,13 +3772,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>891780.0000001139</v>
+        <v>0</v>
       </c>
       <c r="I47" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>891780.0000001139</v>
+        <v>0</v>
       </c>
       <c r="K47" s="6" t="n">
         <v>0</v>
@@ -3800,7 +3796,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="6" t="n">
-        <v>891780.0000001139</v>
+        <v>0</v>
       </c>
       <c r="Q47" s="6" t="n">
         <v>0</v>
@@ -3813,12 +3809,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S31</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
+          <t>Janus Henderson Anemoy Treasury Fund (JTRSY)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3828,7 +3824,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
@@ -3841,13 +3837,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>9.31926637265e-08</v>
+        <v>0</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J48" s="6" t="n">
-        <v>9.31926637265e-08</v>
+        <v>0</v>
       </c>
       <c r="K48" s="6" t="n">
         <v>0</v>
@@ -3856,7 +3852,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N48" s="6" t="n">
         <v>0</v>
@@ -3865,7 +3861,7 @@
         <v>0</v>
       </c>
       <c r="P48" s="6" t="n">
-        <v>9.31926637265e-08</v>
+        <v>0</v>
       </c>
       <c r="Q48" s="6" t="n">
         <v>0</v>
@@ -3873,38 +3869,34 @@
       <c r="R48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S38</t>
+          <t>S21</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>USDS raw (Base — POL)</t>
+          <t>Superstate Short Duration US Government Securities Fund (USTB)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>0</v>
@@ -3922,7 +3914,7 @@
         <v>0</v>
       </c>
       <c r="L49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="M49" s="7" t="n">
         <v>0</v>
@@ -3937,36 +3929,36 @@
         <v>0</v>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="R49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>CoF excluded (already deducted from utilized)</t>
+          <t>SDE (fixed)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S42</t>
+          <t>S22</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
+          <t>Superstate Crypto Carry Fund (USCC)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
@@ -4016,17 +4008,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S44</t>
+          <t>S26</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>USDS raw (Arbitrum — POL)</t>
+          <t>USDC raw (ALM idle)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4035,31 +4027,31 @@
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0</v>
+        <v>891780.0000001139</v>
       </c>
       <c r="I51" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J51" s="6" t="n">
-        <v>0</v>
+        <v>891780.0000001139</v>
       </c>
       <c r="K51" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="M51" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N51" s="6" t="n">
         <v>0</v>
@@ -4068,34 +4060,30 @@
         <v>0</v>
       </c>
       <c r="P51" s="6" t="n">
-        <v>0</v>
+        <v>891780.0000001139</v>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="R51" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S48</t>
+          <t>S31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>USDS raw (Optimism — POL)</t>
+          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4104,28 +4092,28 @@
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="F52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="G52" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>0</v>
+        <v>9.31926637265e-08</v>
       </c>
       <c r="I52" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J52" s="6" t="n">
-        <v>0</v>
+        <v>9.31926637265e-08</v>
       </c>
       <c r="K52" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="M52" s="7" t="n">
         <v>0</v>
@@ -4137,10 +4125,10 @@
         <v>0</v>
       </c>
       <c r="P52" s="6" t="n">
-        <v>0</v>
+        <v>9.31926637265e-08</v>
       </c>
       <c r="Q52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="R52" s="6" t="n">
         <v>0</v>
@@ -4154,17 +4142,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S52</t>
+          <t>S38</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>USDS raw (Unichain — POL)</t>
+          <t>USDS raw (Base — POL)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4173,10 +4161,10 @@
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>89900000</v>
+        <v>65170000</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>89900000</v>
+        <v>65170000</v>
       </c>
       <c r="G53" s="6" t="n">
         <v>0</v>
@@ -4194,7 +4182,7 @@
         <v>0</v>
       </c>
       <c r="L53" s="6" t="n">
-        <v>89900000</v>
+        <v>65170000</v>
       </c>
       <c r="M53" s="7" t="n">
         <v>0</v>
@@ -4209,7 +4197,7 @@
         <v>0</v>
       </c>
       <c r="Q53" s="6" t="n">
-        <v>89900000</v>
+        <v>65170000</v>
       </c>
       <c r="R53" s="6" t="n">
         <v>0</v>
@@ -4223,59 +4211,331 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>S42</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>arbitrum</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>S44</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>USDS raw (Arbitrum — POL)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>arbitrum</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="6" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="M55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="6" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="R55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>S48</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>USDS raw (Optimism — POL)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>optimism</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="M56" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="R56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>S52</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>USDS raw (Unichain — POL)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>unichain</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="G57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="M57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="R57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S54" t="inlineStr">
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S58" t="inlineStr">
         <is>
           <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>

</xml_diff>

<commit_message>
settlements(spark): refresh xlsx with Debt tab + new POL headline rows
Re-running scripts/run_spark_2026.py after PR #118 + post-#117 main
brings two content additions into the Spark xlsx files:

* "Debt" tab (introduced in #117) — daily cum_debt, deductions,
  effective APYs, daily Sky charge. Was already present in Grove
  xlsxes after #117 but Spark hadn't been re-rendered since.
* New headline rows ``pol_agent_rate`` and ``susds_pol_ssr_credit``
  on the Summary tab, matching the summary.md changes.

All numerical differences vs main verified to match the PR's purpose:
prime_agent_revenue and sky_revenue_gross unchanged; sky_revenue (net)
reduced by exactly ``pol_agent_rate + susds_pol_ssr_credit``
(\$22.33M cumulative Jan–May 2026); all other reductions
(susds_spread_reimbursement, curve_susds_spread, psm3_susds_spread)
unchanged.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,6 +88,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -523,7 +525,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>8402460.95851364</v>
+        <v>5927607.895917897</v>
       </c>
     </row>
     <row r="10">
@@ -539,7 +541,7 @@
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="n">
-        <v>8429957.991614142</v>
+        <v>5955104.9290184</v>
       </c>
     </row>
     <row r="13">
@@ -561,7 +563,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>8402460.95851364</v>
+        <v>5927607.895917897</v>
       </c>
     </row>
     <row r="15">
@@ -571,7 +573,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>-2336956.314939647</v>
+        <v>-4811809.377535391</v>
       </c>
     </row>
     <row r="16">
@@ -619,13 +621,13 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>-8402460.95851364</v>
+        <v>-5927607.895917897</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-5517596.021612381</v>
+        <v>-3042742.959016637</v>
       </c>
     </row>
     <row r="25">
@@ -660,7 +662,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-05T12:56:39+00:00</t>
+          <t>2026-06-08T12:35:25+00:00</t>
         </is>
       </c>
     </row>
@@ -816,7 +818,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sUSDS raw / POL (ALM — Cat B 4626, demand-side spread)</t>
+          <t>sUSDS raw / POL (ALM — Cat B 4626, demand-side spread + agent rate)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -857,13 +859,13 @@
         <v>1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>1454465.949905966</v>
+        <v>1030623.123924462</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>1454465.949905966</v>
+        <v>1030623.123924462</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-1454465.949905966</v>
+        <v>-1030623.123924462</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -922,13 +924,13 @@
         <v>1</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>1350618.260706183</v>
+        <v>957037.4687481844</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>1350618.260706183</v>
+        <v>957037.4687481844</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>-1350618.26070619</v>
+        <v>-957037.468748192</v>
       </c>
       <c r="Q3" s="6" t="n">
         <v>0</v>
@@ -987,13 +989,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>946501.8694127946</v>
+        <v>670683.7746993145</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>946501.8694127946</v>
+        <v>670683.7746993145</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>20063.72862020546</v>
+        <v>295881.8233336855</v>
       </c>
       <c r="Q4" s="6" t="n">
         <v>0</v>
@@ -1052,13 +1054,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>703463.9108016299</v>
+        <v>498468.9901921512</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>703463.9108016299</v>
+        <v>498468.9901921512</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>193928.1687364963</v>
+        <v>398923.089345975</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>82530624.22670487</v>
@@ -1121,13 +1123,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>607233.2434632853</v>
+        <v>430280.6967529046</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>607233.2434632853</v>
+        <v>430280.6967529046</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>-1242941.118500961</v>
+        <v>-1065988.571790581</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>0</v>
@@ -1186,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>537098.1921680442</v>
+        <v>380583.5514418185</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>537098.1921680442</v>
+        <v>380583.5514418185</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-1188101.37595719</v>
+        <v>-1031586.735230964</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>0</v>
@@ -1251,13 +1253,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>535349.067247757</v>
+        <v>379344.1352907583</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>535349.067247757</v>
+        <v>379344.1352907583</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>315556.3939936479</v>
+        <v>471561.3259506465</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>0</v>
@@ -1316,13 +1318,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>433980.3659927064</v>
+        <v>307515.0714598725</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>433980.3659927064</v>
+        <v>307515.0714598725</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>-983189.972822314</v>
+        <v>-856724.67828948</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>0</v>
@@ -1381,13 +1383,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>403208.6710770108</v>
+        <v>285710.4906482591</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>403208.6710770108</v>
+        <v>285710.4906482591</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>-164518.8427410108</v>
+        <v>-47020.66231225905</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
@@ -1446,13 +1448,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>282068.8740994219</v>
+        <v>199871.7840077292</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>282068.8740994219</v>
+        <v>199871.7840077292</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>-274637.2155162088</v>
+        <v>-192440.1254245161</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -1511,13 +1513,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>266436.45144477</v>
+        <v>188794.7723582736</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>266436.45144477</v>
+        <v>188794.7723582736</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>191842.059108988</v>
+        <v>269483.7381954844</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>95188953.04035926</v>
@@ -1580,13 +1582,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>232148.8659050326</v>
+        <v>164498.8591242264</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>211209.9879619063</v>
+        <v>143559.9811811001</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>-232148.8659050326</v>
+        <v>-164498.8591242264</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -1645,13 +1647,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>211070.6539832326</v>
+        <v>149563.0040641669</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>192032.9445208107</v>
+        <v>130525.294601745</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>-211070.6539832326</v>
+        <v>-149563.0040641669</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
@@ -1710,13 +1712,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>137288.5466256973</v>
+        <v>97281.58353351145</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>137288.5466256973</v>
+        <v>97281.58353351145</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>80832.91816657386</v>
+        <v>120839.8812587597</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>0</v>
@@ -1775,13 +1777,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>121820.3958662906</v>
+        <v>86320.97365603378</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>121820.3958662906</v>
+        <v>86320.97365603378</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>23672.03626670938</v>
+        <v>59171.45847696622</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>0</v>
@@ -1840,13 +1842,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>121028.5843097249</v>
+        <v>85759.9022194422</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>110112.3011540389</v>
+        <v>74843.61906375624</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>-121028.5843097249</v>
+        <v>-85759.9022194422</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>0</v>
@@ -1859,262 +1861,262 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S18</t>
+          <t>SPREAD</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Arkis Spark Prime USDC 1 (ERC-4626)</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>30bps sUSDS spread (Curve LP + PSM3) — Sky Revenue reduction</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" s="6" t="n">
-        <v>15024030.59441916</v>
+        <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>15106645.23632516</v>
+        <v>0</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>82614.64190600339</v>
+        <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>82614.64190600339</v>
+        <v>0</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>82614.64190600339</v>
+        <v>0</v>
       </c>
       <c r="K18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>15024030.59441916</v>
+        <v>0</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>42378.03913457882</v>
+        <v>0</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>42378.03913457882</v>
+        <v>-39145.45144251771</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>40236.60277142459</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" t="inlineStr"/>
+        <v>39145.45144251771</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>sky-revenue reduction (no CoF; computed outside venue loop)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SPREAD</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>30bps sUSDS spread (Curve LP + PSM3) — Sky Revenue reduction</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+          <t>Arkis Spark Prime USDC 1 (ERC-4626)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="E19" s="6" t="n">
-        <v>0</v>
+        <v>15024030.59441916</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0</v>
+        <v>15106645.23632516</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0</v>
+        <v>82614.64190600339</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0</v>
+        <v>82614.64190600339</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>0</v>
+        <v>82614.64190600339</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0</v>
+        <v>15024030.59441916</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>0</v>
+        <v>30028.74497096095</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>-39145.45144251771</v>
+        <v>30028.74497096095</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>0</v>
+        <v>52585.89693504245</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>39145.45144251771</v>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>sky-revenue reduction (no CoF; computed outside venue loop)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S54</t>
+          <t>S24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aave Avalanche USDC (aAvaUSDC)</t>
+          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>10000438.058711</v>
+        <v>50000864.48440416</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>10000965.036792</v>
+        <v>49999911.74966041</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>526.978081</v>
+        <v>-952.7347437553233</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>31596.950878</v>
+        <v>27497.03310050249</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>31596.950878</v>
+        <v>0</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0</v>
+        <v>27497.03310050249</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>9999435.801524</v>
+        <v>49999946.74995758</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>28205.24619259639</v>
+        <v>0</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>28205.24619259639</v>
+        <v>27497.03310050249</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>3391.704685403611</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>0</v>
+        <v>49999946.74995758</v>
       </c>
       <c r="R20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>SDE (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>S24</t>
+          <t>S54</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
+          <t>Aave Avalanche USDC (aAvaUSDC)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>avalanche_c</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>50000864.48440416</v>
+        <v>10000438.058711</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>49999911.74966041</v>
+        <v>10000965.036792</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>-952.7347437553233</v>
+        <v>526.978081</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>31596.950878</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0</v>
+        <v>31596.950878</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>0</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>49999946.74995758</v>
+        <v>9999435.801524</v>
       </c>
       <c r="M21" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>0</v>
+        <v>19986.0154470798</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>19986.0154470798</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>0</v>
+        <v>11610.9354309202</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>49999946.74995758</v>
+        <v>0</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>SDE (fixed)</t>
-        </is>
-      </c>
+      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2165,13 +2167,13 @@
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>19379.60811033649</v>
+        <v>13732.23776905752</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>19379.60811033649</v>
+        <v>13732.23776905752</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>3534.024676751853</v>
+        <v>9181.395018030822</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2230,13 +2232,13 @@
         <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>14103.92795974866</v>
+        <v>9993.932339510246</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>14103.92795974866</v>
+        <v>9993.932339510246</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>-14103.92795974865</v>
+        <v>-9993.932339510236</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
@@ -2295,13 +2297,13 @@
         <v>1</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>14086.26966065105</v>
+        <v>9981.419807759094</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>14086.26966065105</v>
+        <v>9981.419807759094</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>-14086.26966064621</v>
+        <v>-9981.419807754255</v>
       </c>
       <c r="Q24" s="6" t="n">
         <v>0</v>
@@ -2360,13 +2362,13 @@
         <v>1</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>14049.00025329229</v>
+        <v>9955.010999054168</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>14049.00025329229</v>
+        <v>9955.010999054168</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>-14049.00025329063</v>
+        <v>-9955.010999052509</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -2425,13 +2427,13 @@
         <v>1</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>13958.2012234117</v>
+        <v>9890.671521164773</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>13958.2012234117</v>
+        <v>9890.671521164773</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>-13958.20122351087</v>
+        <v>-9890.671521263952</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>0</v>
@@ -2490,13 +2492,13 @@
         <v>1</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>2736.56568805195</v>
+        <v>1939.108906899427</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>2489.738658757273</v>
+        <v>1692.281877604751</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>-2736.56568805195</v>
+        <v>-1939.108906899427</v>
       </c>
       <c r="Q27" s="6" t="n">
         <v>0</v>
@@ -2555,13 +2557,13 @@
         <v>1</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>60.5412987642022</v>
+        <v>42.8990877805288</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>60.5412987642022</v>
+        <v>42.8990877805288</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>-774.9161127668142</v>
+        <v>-757.2739017831408</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>0</v>
@@ -2620,13 +2622,13 @@
         <v>1</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>4.595926479553287</v>
+        <v>3.25663732862952</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>4.595926479553287</v>
+        <v>3.25663732862952</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>-4.595926480113287</v>
+        <v>-3.256637329189521</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -2685,13 +2687,13 @@
         <v>1</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>0.8873810435980858</v>
+        <v>0.6287912228701786</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>0.8873810435980858</v>
+        <v>0.6287912228701786</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>1.491002180420111</v>
+        <v>1.749592001148018</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>0</v>
@@ -2750,13 +2752,13 @@
         <v>1</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>0.8007843598651403</v>
+        <v>0.5674294943841202</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>0.8007843598651403</v>
+        <v>0.5674294943841202</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.8007843598651403</v>
+        <v>-0.5674294943841202</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>0</v>
@@ -2815,13 +2817,13 @@
         <v>1</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>0.2770438751272927</v>
+        <v>0.1963111092881128</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0.2770438751272927</v>
+        <v>0.1963111092881128</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.1115362422753438</v>
+        <v>0.1922690081145236</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -2880,13 +2882,13 @@
         <v>1</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>0.1787808553252768</v>
+        <v>0.1266827068898633</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>0.1787808553252768</v>
+        <v>0.1266827068898633</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>-0.1787808544202768</v>
+        <v>-0.1266827059848633</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -2945,13 +2947,13 @@
         <v>1</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>0.0617605599461623</v>
+        <v>0.04376304665719607</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>0.0617605599461623</v>
+        <v>0.04376304665719607</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.06079052886814793</v>
+        <v>-0.04279301557918169</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>0</v>
@@ -3010,13 +3012,13 @@
         <v>1</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>0.00313405608637691</v>
+        <v>0.002220767474484412</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>0.00313405608637691</v>
+        <v>0.002220767474484412</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>0.09635194391362309</v>
+        <v>0.09726523252551558</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -3075,13 +3077,13 @@
         <v>1</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>0.0001612782354488736</v>
+        <v>0.0001142804882094966</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>0.0001612782354488736</v>
+        <v>0.0001142804882094966</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>1.572176455112641e-05</v>
+        <v>6.271951179050342e-05</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>0</v>
@@ -3140,13 +3142,13 @@
         <v>1</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.775338359681708e-05</v>
+        <v>1.257990787887737e-05</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>1.775338359681708e-05</v>
+        <v>1.257990787887737e-05</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>-1.753383596817084e-06</v>
+        <v>3.420092121122629e-06</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>0</v>
@@ -3205,13 +3207,13 @@
         <v>1</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>1.61776273567708e-05</v>
+        <v>1.146333941004181e-05</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>1.61776273567708e-05</v>
+        <v>1.146333941004181e-05</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>-1.21644138284758e-05</v>
+        <v>-7.450125881746809e-06</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>0</v>
@@ -3270,13 +3272,13 @@
         <v>1</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>4.744390087360396e-06</v>
+        <v>3.361837472556679e-06</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>4.744390087360396e-06</v>
+        <v>3.361837472556679e-06</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>1.255609912639604e-06</v>
+        <v>2.638162527443321e-06</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -3335,13 +3337,13 @@
         <v>1</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>3.498055934399643e-06</v>
+        <v>2.478694901731143e-06</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>3.498055934399643e-06</v>
+        <v>2.478694901731143e-06</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>-3.498055934399643e-06</v>
+        <v>-2.478694901731143e-06</v>
       </c>
       <c r="Q40" s="6" t="n">
         <v>0</v>
@@ -3400,13 +3402,13 @@
         <v>1</v>
       </c>
       <c r="N41" s="6" t="n">
-        <v>8.160893161715145e-07</v>
+        <v>5.782744659566913e-07</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>8.160893161715145e-07</v>
+        <v>5.782744659566913e-07</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>-3.267373086345146e-07</v>
+        <v>-8.892245841969127e-08</v>
       </c>
       <c r="Q41" s="6" t="n">
         <v>0</v>
@@ -3465,13 +3467,13 @@
         <v>1</v>
       </c>
       <c r="N42" s="6" t="n">
-        <v>2.112587092447954e-07</v>
+        <v>1.496962585423173e-07</v>
       </c>
       <c r="O42" s="6" t="n">
-        <v>2.112587092447954e-07</v>
+        <v>1.496962585423173e-07</v>
       </c>
       <c r="P42" s="6" t="n">
-        <v>-2.112587092447954e-07</v>
+        <v>-1.496962585423173e-07</v>
       </c>
       <c r="Q42" s="6" t="n">
         <v>0</v>
@@ -3530,13 +3532,13 @@
         <v>1</v>
       </c>
       <c r="N43" s="6" t="n">
-        <v>2.043056587295296e-10</v>
+        <v>1.447693816750306e-10</v>
       </c>
       <c r="O43" s="6" t="n">
-        <v>2.043056587295296e-10</v>
+        <v>1.447693816750306e-10</v>
       </c>
       <c r="P43" s="6" t="n">
-        <v>-1.088917746587295e-07</v>
+        <v>-1.08832238381675e-07</v>
       </c>
       <c r="Q43" s="6" t="n">
         <v>0</v>
@@ -4585,7 +4587,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>8402460.95851364</v>
+        <v>5927607.895917897</v>
       </c>
     </row>
     <row r="5">
@@ -4605,7 +4607,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>8429957.991614142</v>
+        <v>5955104.9290184</v>
       </c>
     </row>
     <row r="8">
@@ -4632,7 +4634,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>8402460.95851364</v>
+        <v>5927607.895917897</v>
       </c>
     </row>
     <row r="12">
@@ -4642,7 +4644,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>-2336956.314939647</v>
+        <v>-4811809.377535391</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
@@ -4937,4 +4939,1669 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Daily ilk debt + Sky charge breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40). utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>cum_debt</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>− ALM idle</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>− PSM USDS</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>− SDE NAV</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>− Curve idle</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>− Lending idle</t>
+        </is>
+      </c>
+      <c r="H5" s="2">
+        <f> utilized</f>
+        <v/>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>SSR APY</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>base APY</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>T (months)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>ref_rate APY</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>sub APY</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>daily Sky charge</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>daily Sky charge (gross on cum_debt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>2980874080.901297</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>-35631246.89117327</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>61155231.42517054</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>68023908.80789006</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>136523837.3994096</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>2415832350.16</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>279433.4611766197</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>344790.4659869125</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>3000048459.330918</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>-35324494.46188942</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>57960012.56082956</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>63910342.76190185</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>139968910.2863361</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>2438563688.18374</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>282062.7398435473</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>347008.3197755434</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>2996569482.922088</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>-35640122.57323464</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>58249830.75246512</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>59098488.77875964</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>141176296.2006703</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>2438714989.763428</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>282080.2405298391</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>346605.9150229095</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>3022609460.527921</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>-35870148.56141944</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>57014923.37279677</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>59983836.46674705</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>148508144.6309396</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>2458002704.618857</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>284311.2036676095</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>349617.8959953795</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>3019382604.232045</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>-35449106.54717439</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>25866980.28616193</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>57800282.28988203</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>149471285.1063189</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>2486723163.096857</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>287633.2293531068</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>349244.6533639459</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>2989159888.02578</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>-26512889.94736019</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>57425219.16937209</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>58767695.27812117</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>149868749.0652394</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>2414641114.460408</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>279295.673836123</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>345748.8651752017</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>3005104832.398945</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>-22215108.56536281</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>60341365.99153879</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>51918769.71159481</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>147757637.4539552</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>2432332167.807219</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>281341.9550146296</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>347593.1781690927</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>3124011111.461903</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>-19566817.34517212</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>60420720.77145881</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>56911097.03338878</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>178672791.4909193</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>2512603319.511308</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>290626.7241964901</v>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>361346.7787084657</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>2960713599.183378</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>-18904509.07902374</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>60988618.38742205</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>55649780.79160649</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>180832999.7715634</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>2347176709.31181</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>271492.2299275895</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>342458.5520256424</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>2929332071.555636</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>-18457985.85961093</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>61046384.58909018</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>56775902.51711459</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>180850061.4698032</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>2314147708.839239</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>267671.8456527272</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>338828.72693391</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>2915887950.247579</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>-17784002.55402869</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>61276478.31621934</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>56127466.01608274</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>180948176.0627011</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>2300349832.406604</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>266075.8787934363</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>337273.6780707967</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>2923094023.443971</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>-16987680.02863479</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>60668020.63561259</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>56752870.53974199</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>192300906.7246515</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>2295389905.5726</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>265502.1761015599</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>338107.1870577206</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>2857933671.340444</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>-16857926.75909428</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>57160001.80819702</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>64864210.75065267</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>188233620.1097723</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>2229563765.430916</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>257888.2263279055</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>330570.2473695962</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>2777967078.343399</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>-16653002.95647965</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>26467496.09842381</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>64724055.24673219</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>166180609.8119938</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>2202277920.142729</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>254732.1388661646</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>321320.7057537691</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>2761558411.996649</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>-15886136.17797409</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>52083103.27887755</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>56217051.11037463</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>167989632.8234313</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>2166184760.96194</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>250557.3307947276</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>319422.7551653266</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>2763461890.012003</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>-15043862.03899061</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>56966377.49472634</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>56877842.42658328</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>168333690.2034414</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>2161357841.926242</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>249999.0127918766</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>319642.9258448312</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>2762476728.292931</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>-15022654.2587271</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>56722765.30750743</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>54150921.01912522</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>168377058.241571</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>2163278637.983454</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M22" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>250221.1866072267</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>319528.9745812177</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>2764448889.752242</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>-12733132.44335289</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>56314463.29144242</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>53051083.27470047</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>168436868.059635</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>2164409607.569817</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>250352.0031127602</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>319757.0897078894</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>3102663227.213934</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>16536515.46810593</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>58628042.5439949</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>56394358.092057</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>168524717.3268149</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>2467609593.782961</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M24" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>285422.4092072191</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>358877.5207801113</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>3082931716.306114</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>16553539.76078879</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>61079686.83723351</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>52581006.50545063</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>167762562.2180895</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>2449984920.984551</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M25" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>283383.8061055433</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>356595.2248307043</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>2991178521.440929</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>17726279.73006013</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>60040981.97034811</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>47705185.04519594</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>171079753.1258666</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>2359656321.569458</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M26" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>272935.7163711194</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>345982.3556001497</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>3010068465.358339</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>19330251.24530254</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>60247556.90564181</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>56980214.65006325</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>176370776.497611</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>2362169666.059721</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M27" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>273226.4288247367</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>348167.3095394926</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>3033644440.628436</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>24317881.0827431</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>60932295.74696831</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>62602403.61620532</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>183037062.7820338</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>2367784797.400486</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M28" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>273875.9174307682</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>350894.2853455336</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>3035101444.900412</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>29923107.73851411</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>61469915.64923963</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>64210065.47836063</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>181882100.6903611</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>2362646255.343936</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M29" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>273281.5547498611</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>351062.813491388</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>3045163199.614203</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>33035630.50479232</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>60828676.08782978</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>62772546.87581208</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>182325188.4918531</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>2371231157.653916</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M30" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>274274.5495519143</v>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>352226.6322245044</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>3066394900.887817</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>32641339.83210305</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>60384722.42316125</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>55182340.31570686</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>190865757.8391129</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>2392350740.477733</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>276717.4004089593</v>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>354682.4515503616</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>3105785729.944945</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>33467761.63995818</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>61004518.25471943</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>61060793.97157621</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>203149752.3525293</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>2412132903.726162</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M32" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>279005.555191597</v>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>359238.693088116</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>3127285444.151954</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>33745745.65885227</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>61253989.62770834</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>67839079.21769939</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>207053370.3424328</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>2422423259.305261</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M33" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>280195.8156316542</v>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>361725.5128191187</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>3256628917.902534</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>33939394.27332065</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>61643050.05621564</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>53880998.6091714</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>243793315.2617481</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>2528402159.702078</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M34" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>292454.1376744125</v>
+      </c>
+      <c r="O34" s="3" t="n">
+        <v>376686.358321638</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>3239542238.123795</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>34179027.74470039</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>61589076.04808185</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>55051048.5469578</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>244460552.884327</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>2509292532.899728</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M35" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>290243.7735492609</v>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>374709.9835660498</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>3196239124.626659</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>334970000</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>34415630.20183328</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>60987052.30967253</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>54786694.01177735</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>234570710.5538552</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>2476509037.54952</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J36" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="M36" s="7" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>286451.7862557017</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>369701.2175879689</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Σ daily charges</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" s="10" t="n">
+        <v>8492746.107546687</v>
+      </c>
+      <c r="O38" s="10" t="n">
+        <v>10739417.27345329</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
settlements(spark): re-render Jan–May 2026 with reconciliation note
Refresh after review-fix `e65030f`. Adds the aggregated VSR-liability
reconciliation row under the position-only sub-section in each xlsx
"Venues" tab + ``summary.md``. Numbers unchanged at the prime level
(``prime_agent_revenue`` / ``sky_revenue`` byte-identical).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -75,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,6 +85,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -662,7 +663,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-08T16:50:50+00:00</t>
+          <t>2026-06-08T17:07:07+00:00</t>
         </is>
       </c>
     </row>
@@ -689,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S61"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4434,6 +4435,20 @@
         <v>95656876.179346</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Aggregated actual_revenue (included in prime_agent_revenue, not in Venues body above)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" s="9" t="n">
+        <v>-1836635.040470432</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4539,14 +4554,14 @@
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Note: sky_revenue can EXCEED sky_revenue_gross for primes with active SDE positions — sky_revenue also adds sde_revenue on top of BR-on-utilized. The subsidised BR (ref_rate ramp) is already applied here; this is NOT the raw Maker base rate.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>sUSDS spread (Curve LP + PSM3) — 30 bps × value × n_days credited to prime_agent_revenue. Sky still charges full BR on the underlying utilized; this row is the prime's offsetting pickup on the share-price-appreciation accounting (SSR + BR + 30 bps nets to zero economically).</t>
         </is>
@@ -4866,7 +4881,7 @@
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40). utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
         </is>
@@ -6485,10 +6500,10 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="10" t="n">
+      <c r="N38" s="11" t="n">
         <v>8492746.107546687</v>
       </c>
-      <c r="O38" s="10" t="n">
+      <c r="O38" s="11" t="n">
         <v>10739417.27345329</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(spark): hide per-venue PnL for Savings V2 vaults (#120)
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -75,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,6 +85,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -662,7 +663,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-08T14:48:42+00:00</t>
+          <t>2026-06-08T17:07:07+00:00</t>
         </is>
       </c>
     </row>
@@ -689,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S58"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4225,47 +4226,39 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S56</t>
+          <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Spark Savings V2 — spUSDC vault</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
+          <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
       <c r="E54" s="6" t="n">
-        <v>215278739.036717</v>
+        <v>0</v>
       </c>
       <c r="F54" s="6" t="n">
-        <v>207131500.431691</v>
+        <v>0</v>
       </c>
       <c r="G54" s="6" t="n">
-        <v>-8147238.605026</v>
+        <v>0</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>-635707.8750376763</v>
+        <v>0</v>
       </c>
       <c r="I54" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J54" s="6" t="n">
-        <v>-635707.8750376763</v>
+        <v>0</v>
       </c>
       <c r="K54" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L54" s="6" t="n">
-        <v>215278739.036717</v>
+        <v>0</v>
       </c>
       <c r="M54" s="7" t="n">
         <v>0</v>
@@ -4277,7 +4270,7 @@
         <v>0</v>
       </c>
       <c r="P54" s="6" t="n">
-        <v>-635707.8750376763</v>
+        <v>0</v>
       </c>
       <c r="Q54" s="6" t="n">
         <v>0</v>
@@ -4287,276 +4280,173 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>CoF excluded (Savings V2 depositor capital; not in cum_alm_usds)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>S57</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spUSDT vault</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="n">
-        <v>153856441.430568</v>
-      </c>
-      <c r="F55" s="6" t="n">
-        <v>120038508.359851</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>-33817933.070717</v>
-      </c>
-      <c r="H55" s="6" t="n">
-        <v>-549209.6068296075</v>
-      </c>
-      <c r="I55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="6" t="n">
-        <v>-549209.6068296075</v>
-      </c>
-      <c r="K55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" s="6" t="n">
-        <v>153856441.430568</v>
-      </c>
-      <c r="M55" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" s="6" t="n">
-        <v>-549209.6068296075</v>
-      </c>
-      <c r="Q55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>CoF excluded (Savings V2 depositor capital; not in cum_alm_usds)</t>
+          <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>S59</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spPYUSD vault</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="n">
-        <v>21463.341472</v>
-      </c>
-      <c r="F56" s="6" t="n">
-        <v>285387.136685</v>
-      </c>
-      <c r="G56" s="6" t="n">
-        <v>263923.795213</v>
-      </c>
-      <c r="H56" s="6" t="n">
-        <v>-714.374814002612</v>
-      </c>
-      <c r="I56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="6" t="n">
-        <v>-714.374814002612</v>
-      </c>
-      <c r="K56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="6" t="n">
-        <v>21463.341472</v>
-      </c>
-      <c r="M56" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="6" t="n">
-        <v>-714.374814002612</v>
-      </c>
-      <c r="Q56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S56" t="inlineStr">
-        <is>
-          <t>CoF excluded (Savings V2 depositor capital; not in cum_alm_usds)</t>
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>Position-only venues (PnL aggregated at prime level)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>S60</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spUSDC vault (Avalanche-C, CREATE2 same address)</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>avalanche_c</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>190414182.348414</v>
-      </c>
-      <c r="F57" s="6" t="n">
-        <v>95656876.179346</v>
-      </c>
-      <c r="G57" s="6" t="n">
-        <v>-94757306.16906799</v>
-      </c>
-      <c r="H57" s="6" t="n">
-        <v>-651003.1837891456</v>
-      </c>
-      <c r="I57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" s="6" t="n">
-        <v>-651003.1837891456</v>
-      </c>
-      <c r="K57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" s="6" t="n">
-        <v>190414182.348414</v>
-      </c>
-      <c r="M57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" s="6" t="n">
-        <v>-651003.1837891456</v>
-      </c>
-      <c r="Q57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>CoF excluded (Savings V2 depositor capital; not in cum_alm_usds)</t>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Venue</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Pricing cat.</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Position SoM</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Position EoM</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PSM_CURVE_DEDUCT</t>
+          <t>S56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
+          <t>Spark Savings V2 — spUSDC vault</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
       <c r="E58" s="6" t="n">
-        <v>0</v>
+        <v>215278739.036717</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M58" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S58" t="inlineStr">
-        <is>
-          <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
-        </is>
+        <v>207131500.431691</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>S57</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spUSDT vault</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>153856441.430568</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>120038508.359851</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>S59</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spPYUSD vault</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>21463.341472</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>285387.136685</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>S60</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spUSDC vault (Avalanche-C, CREATE2 same address)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>avalanche_c</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>190414182.348414</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>95656876.179346</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Aggregated actual_revenue (included in prime_agent_revenue, not in Venues body above)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" s="9" t="n">
+        <v>-1836635.040470432</v>
       </c>
     </row>
   </sheetData>
@@ -4664,14 +4554,14 @@
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Note: sky_revenue can EXCEED sky_revenue_gross for primes with active SDE positions — sky_revenue also adds sde_revenue on top of BR-on-utilized. The subsidised BR (ref_rate ramp) is already applied here; this is NOT the raw Maker base rate.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>sUSDS spread (Curve LP + PSM3) — 30 bps × value × n_days credited to prime_agent_revenue. Sky still charges full BR on the underlying utilized; this row is the prime's offsetting pickup on the share-price-appreciation accounting (SSR + BR + 30 bps nets to zero economically).</t>
         </is>
@@ -4991,7 +4881,7 @@
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40). utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
         </is>
@@ -6610,10 +6500,10 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="10" t="n">
+      <c r="N38" s="11" t="n">
         <v>8492746.107546687</v>
       </c>
-      <c r="O38" s="10" t="n">
+      <c r="O38" s="11" t="n">
         <v>10739417.27345329</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: regenerate settlements on fix/savings-v2-excluded-from-prime-revenue
Re-ran scripts/run_grove_2026.py, run_spark_2026.py, run_obex_2026.py
on the current branch head. xlsx + summary.md refreshed for all 3
primes × 5 months (Jan–May 2026).

Spark May 2026 prime_agent_revenue = $12,636,329.49 (full headline
under the savings-v2-excluded scope; Position-only venues note
included where appropriate).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>2975150.085934307</v>
+        <v>4811785.126404739</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>3081542.631057669</v>
+        <v>4918177.671528101</v>
       </c>
     </row>
     <row r="8">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>2975150.085934307</v>
+        <v>4811785.126404739</v>
       </c>
     </row>
     <row r="22">
@@ -628,7 +628,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-5429826.797119002</v>
+        <v>-3593191.75664857</v>
       </c>
     </row>
     <row r="25">
@@ -663,7 +663,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-09T16:56:30+00:00</t>
+          <t>2026-06-09T22:27:02+00:00</t>
         </is>
       </c>
     </row>
@@ -4446,7 +4446,7 @@
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" s="9" t="n">
-        <v>-1836635.040470432</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(spark): exclude Savings V2 vaults from prime_agent_revenue (#126)
Co-authored-by: Cursor <cursoragent@cursor.com>
Co-authored-by: Claude <claude@no-reply.invalid>
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
Co-authored-by: lakonema2000 <lakonema2000@gmail.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>2975150.085934307</v>
+        <v>4811785.126404739</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>3081542.631057669</v>
+        <v>4918177.671528101</v>
       </c>
     </row>
     <row r="8">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>2975150.085934307</v>
+        <v>4811785.126404739</v>
       </c>
     </row>
     <row r="22">
@@ -628,7 +628,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-5429826.797119002</v>
+        <v>-3593191.75664857</v>
       </c>
     </row>
     <row r="25">
@@ -663,7 +663,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-09T16:56:30+00:00</t>
+          <t>2026-06-09T22:27:02+00:00</t>
         </is>
       </c>
     </row>
@@ -4446,7 +4446,7 @@
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" s="9" t="n">
-        <v>-1836635.040470432</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: re-render settlements after assetsOutstanding carve-out fix
Spark profit +~$31K/month (Σ +$156,718 Jan–May → +$7,625,174); sky
revenue identical to the cent. Grove/OBEX summaries byte-identical
(xlsx re-render only).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7469989.539199479</v>
+        <v>7503304.54830196</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>7576382.084322841</v>
+        <v>7609697.093425322</v>
       </c>
     </row>
     <row r="8">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>7469989.539199479</v>
+        <v>7503304.54830196</v>
       </c>
     </row>
     <row r="22">
@@ -628,7 +628,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-1828595.487782908</v>
+        <v>-1795280.478680426</v>
       </c>
     </row>
     <row r="25">
@@ -663,7 +663,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-10T09:48:50+00:00</t>
+          <t>2026-06-10T10:53:32+00:00</t>
         </is>
       </c>
     </row>
@@ -842,13 +842,13 @@
         <v>-136047042.8806877</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>1100659.67820387</v>
+        <v>1133974.687306352</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>1100659.67820387</v>
+        <v>1133974.687306352</v>
       </c>
       <c r="K2" s="6" t="n">
         <v>0</v>
@@ -866,7 +866,7 @@
         <v>1768020.22891697</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-667360.5507130998</v>
+        <v>-634045.5416106181</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix(spark): book sUSDS SSR + fix Anchorage tranche misclassification — Spark Jan–May PnL −$23.4M → +$7.6M (#130)
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4811785.126404739</v>
+        <v>7503304.54830196</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>4918177.671528101</v>
+        <v>7609697.093425322</v>
       </c>
     </row>
     <row r="8">
@@ -536,13 +536,13 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>27497.03310050249</v>
+        <v>2023.079289802219</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="n">
-        <v>8311142.173643176</v>
+        <v>8285668.219832476</v>
       </c>
     </row>
     <row r="13">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>4811785.126404739</v>
+        <v>7503304.54830196</v>
       </c>
     </row>
     <row r="22">
@@ -628,7 +628,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-3593191.75664857</v>
+        <v>-1795280.478680426</v>
       </c>
     </row>
     <row r="25">
@@ -663,7 +663,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-09T23:14:04+00:00</t>
+          <t>2026-06-10T10:53:32+00:00</t>
         </is>
       </c>
     </row>
@@ -842,13 +842,13 @@
         <v>-136047042.8806877</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>0</v>
+        <v>1133974.687306352</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>0</v>
+        <v>1133974.687306352</v>
       </c>
       <c r="K2" s="6" t="n">
         <v>0</v>
@@ -866,7 +866,7 @@
         <v>1768020.22891697</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-1768020.22891697</v>
+        <v>-634045.5416106181</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -1370,13 +1370,13 @@
         <v>196085966.8971079</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0</v>
+        <v>253276.0568678948</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0</v>
+        <v>253276.0568678948</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>0</v>
@@ -1394,7 +1394,7 @@
         <v>261256.7218003855</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>-282195.5997435118</v>
+        <v>-28919.54287561706</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
@@ -1435,13 +1435,13 @@
         <v>249678.5924484764</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0</v>
+        <v>249678.5924484764</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0</v>
+        <v>249678.5924484764</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>0</v>
@@ -1459,7 +1459,7 @@
         <v>237535.6300490435</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>-256573.3395114655</v>
+        <v>-6894.747062989017</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -1630,13 +1630,13 @@
         <v>100136734.7818235</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0</v>
+        <v>132270.8635847951</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0</v>
+        <v>132270.8635847951</v>
       </c>
       <c r="K14" s="6" t="n">
         <v>0</v>
@@ -1654,7 +1654,7 @@
         <v>136203.6857584099</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>-147119.9689140958</v>
+        <v>-14849.10532930069</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
@@ -1858,12 +1858,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S24</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
+          <t>Spark Blue Chip USDC Vault (Morpho)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1873,113 +1873,109 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>50000864.48440416</v>
+        <v>10124757.36060807</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>49999911.74966041</v>
+        <v>976334.4376037563</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-952.7347437553233</v>
+        <v>-9148422.923004312</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>22913.63278708834</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0</v>
+        <v>22913.63278708834</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>0</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>49999946.74995758</v>
+        <v>6870535.567559426</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>0</v>
+        <v>23557.47081585065</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>23557.47081585065</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>0</v>
+        <v>-643.8380287623078</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>49999946.74995758</v>
+        <v>0</v>
       </c>
       <c r="R18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>SDE (fixed)</t>
-        </is>
-      </c>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S53</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Spark Blue Chip USDC Vault (Morpho)</t>
+          <t>USDC raw (Unichain — ALM idle)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>unichain</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>10124757.36060807</v>
+        <v>5000000</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>976334.4376037563</v>
+        <v>5000000</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>-9148422.923004312</v>
+        <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>22913.63278708834</v>
+        <v>8e-12</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>22913.63278708834</v>
+        <v>8e-12</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>6870535.567559426</v>
+        <v>5000180.50613029</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>23557.47081585065</v>
+        <v>17144.45769021642</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>23557.47081585065</v>
+        <v>17144.45769021642</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>-643.8380287623078</v>
+        <v>-17144.45769021642</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -1992,17 +1988,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S53</t>
+          <t>S45</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>USDC raw (Unichain — ALM idle)</t>
+          <t>USDC raw (Arbitrum — ALM idle)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2014,37 +2010,37 @@
         <v>5000000</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>5000000</v>
+        <v>4994817.315553</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0</v>
+        <v>-5182.684447</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>8e-12</v>
+        <v>4.83813e-09</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>8e-12</v>
+        <v>4.83813e-09</v>
       </c>
       <c r="K20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>5000180.50613029</v>
+        <v>4993920.215864256</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>17144.45769021642</v>
+        <v>17122.99260881328</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>17144.45769021642</v>
+        <v>17122.99260881328</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>-17144.45769021642</v>
+        <v>-17122.99260880844</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -2057,17 +2053,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>S45</t>
+          <t>S49</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>USDC raw (Arbitrum — ALM idle)</t>
+          <t>USDC raw (Optimism — ALM idle)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>optimism</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2079,37 +2075,37 @@
         <v>5000000</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>4994817.315553</v>
+        <v>5000000</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>-5182.684447</v>
+        <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>4.83813e-09</v>
+        <v>1.658e-09</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>4.83813e-09</v>
+        <v>1.658e-09</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>4993920.215864256</v>
+        <v>4980707.317678578</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>17122.99260881328</v>
+        <v>17077.68864955986</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>17122.99260881328</v>
+        <v>17077.68864955986</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-17122.99260880844</v>
+        <v>-17077.6886495582</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>0</v>
@@ -2122,17 +2118,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S49</t>
+          <t>S39</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>USDC raw (Optimism — ALM idle)</t>
+          <t>USDC raw (Base — ALM idle)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2141,40 +2137,40 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>5000000</v>
+        <v>4732058.263226</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>5000000</v>
+        <v>4979093.435761</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0</v>
+        <v>247035.172535</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1.658e-09</v>
+        <v>-9.9179e-08</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>1.658e-09</v>
+        <v>-9.9179e-08</v>
       </c>
       <c r="K22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>4980707.317678578</v>
+        <v>4948516.885305397</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>17077.68864955986</v>
+        <v>16967.31513300877</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>17077.68864955986</v>
+        <v>16967.31513300877</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>-17077.6886495582</v>
+        <v>-16967.31513310795</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2187,132 +2183,136 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S39</t>
+          <t>S51</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>USDC raw (Base — ALM idle)</t>
+          <t>Savings USDS / sUSDS proxy (Unichain — POL)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>unichain</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>4732058.263226</v>
+        <v>970178.1267029551</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>4979093.435761</v>
+        <v>973415.2506528809</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>247035.172535</v>
+        <v>3237.123949925721</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>-9.9179e-08</v>
+        <v>3237.123949925721</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>-9.9179e-08</v>
+        <v>3237.123949925721</v>
       </c>
       <c r="K23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>4948516.885305397</v>
+        <v>970178.1267029551</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16967.31513300877</v>
+        <v>3326.5154777592</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>16967.31513300877</v>
+        <v>3079.688448464524</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>-16967.31513310795</v>
+        <v>-89.39152783347872</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>0</v>
+        <v>246.8270292946761</v>
       </c>
       <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S51</t>
+          <t>S24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Unichain — POL)</t>
+          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>970178.1267029551</v>
+        <v>50000864.48440416</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>973415.2506528809</v>
+        <v>49999911.74966041</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>3237.123949925721</v>
+        <v>-952.7347437553233</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0</v>
+        <v>2023.079289802219</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>0</v>
+        <v>25473.95381070027</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0</v>
+        <v>25473.95381070027</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>0</v>
+        <v>2023.079289802219</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>970178.1267029551</v>
+        <v>49999946.74995758</v>
       </c>
       <c r="M24" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>3326.5154777592</v>
+        <v>0</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>3079.688448464524</v>
+        <v>2023.079289802219</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>-3326.5154777592</v>
+        <v>25473.95381070027</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>0</v>
+        <v>49999946.74995758</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>246.8270292946761</v>
-      </c>
-      <c r="S24" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>SDE (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4503,7 +4503,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>27497.03310050249</v>
+        <v>2023.079289802219</v>
       </c>
     </row>
     <row r="6">
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>8311142.173643176</v>
+        <v>8285668.219832476</v>
       </c>
     </row>
     <row r="8">
@@ -4836,10 +4836,10 @@
         </is>
       </c>
       <c r="I5" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>2023.079289802219</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>27497.03310050249</v>
+        <v>2023.079289802219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: remove agent rate on sUSDS_POL
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="10">
@@ -545,7 +545,7 @@
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="n">
-        <v>7736693.016977214</v>
+        <v>7824194.465170181</v>
       </c>
     </row>
     <row r="13">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="15">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>-2942380.297009195</v>
+        <v>-2854878.848816229</v>
       </c>
     </row>
     <row r="16">
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>-7734669.938868322</v>
+        <v>-7822171.387061289</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-1246305.303708494</v>
+        <v>-1333806.751901461</v>
       </c>
     </row>
     <row r="25">
@@ -666,7 +666,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-23T21:42:32+00:00</t>
+          <t>2026-06-25T11:40:59+00:00</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sUSDS raw / POL (ALM — Cat B 4626, demand-side spread + agent rate)</t>
+          <t>sUSDS raw / POL (ALM — Cat B 4626, demand-side spread)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -863,13 +863,13 @@
         <v>1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>1652541.117523931</v>
+        <v>1670947.3942594</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>1652541.117523931</v>
+        <v>1670947.3942594</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-518566.4581009091</v>
+        <v>-536972.7348363776</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -928,13 +928,13 @@
         <v>1</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>1534551.022002216</v>
+        <v>1551643.105506916</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>1534551.022002216</v>
+        <v>1551643.105506916</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>-1534551.022002223</v>
+        <v>-1551643.105506923</v>
       </c>
       <c r="Q3" s="6" t="n">
         <v>0</v>
@@ -993,13 +993,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>1075400.3949828</v>
+        <v>1087378.382738496</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>1075400.3949828</v>
+        <v>1087378.382738496</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>-108834.7969498004</v>
+        <v>-120812.7847054962</v>
       </c>
       <c r="Q4" s="6" t="n">
         <v>0</v>
@@ -1058,13 +1058,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>799264.5254906372</v>
+        <v>808166.8661858366</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>799264.5254906372</v>
+        <v>808166.8661858366</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>98127.554047489</v>
+        <v>89225.2133522896</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>82530624.22670487</v>
@@ -1127,13 +1127,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>608255.1096587715</v>
+        <v>615029.9558368304</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>608255.1096587715</v>
+        <v>615029.9558368304</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>242650.3515826334</v>
+        <v>235875.5054045745</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>0</v>
@@ -1192,13 +1192,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>458119.2897228166</v>
+        <v>463221.8982661542</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>458119.2897228166</v>
+        <v>463221.8982661542</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-219429.4613868165</v>
+        <v>-224532.0699301542</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>0</v>
@@ -1257,13 +1257,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>320482.1759169488</v>
+        <v>324051.7594850424</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>320482.1759169488</v>
+        <v>324051.7594850424</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-313050.5173337357</v>
+        <v>-316620.1009018293</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>0</v>
@@ -1322,13 +1322,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>302720.865516389</v>
+        <v>306092.6206668108</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>302720.865516389</v>
+        <v>306092.6206668108</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>155557.645037369</v>
+        <v>152185.8898869471</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>95188953.04035926</v>
@@ -1391,13 +1391,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>263763.8552620765</v>
+        <v>266701.7007784666</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>242824.9773189502</v>
+        <v>245762.8228353402</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>-10487.79839418177</v>
+        <v>-13425.6439105718</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
@@ -1456,13 +1456,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>239815.1255672291</v>
+        <v>242486.2261648078</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>220777.4161048071</v>
+        <v>223448.5167023858</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>9863.46688124739</v>
+        <v>7192.366283668689</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -1521,13 +1521,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>155985.0667378869</v>
+        <v>157722.4542525044</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>155985.0667378869</v>
+        <v>157722.4542525044</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>62136.39805438424</v>
+        <v>60399.01053976677</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>0</v>
@@ -1586,13 +1586,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>138410.399456311</v>
+        <v>139952.0374152363</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>138410.399456311</v>
+        <v>139952.0374152363</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>7082.032676688972</v>
+        <v>5540.394717763749</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -1651,13 +1651,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>137510.7557385326</v>
+        <v>139042.3733166896</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>126594.4725828467</v>
+        <v>128126.0901610037</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>-5239.892153737481</v>
+        <v>-6771.509731894468</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
@@ -1777,13 +1777,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>48149.2551643835</v>
+        <v>48685.54954505841</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>48149.2551643835</v>
+        <v>48685.54954505841</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>34465.38674161991</v>
+        <v>33929.09236094499</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>0</v>
@@ -1842,13 +1842,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>32046.35286660667</v>
+        <v>32403.29045379908</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>32046.35286660667</v>
+        <v>32403.29045379908</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>-449.4019886066722</v>
+        <v>-806.3395757990797</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>0</v>
@@ -1907,13 +1907,13 @@
         <v>1</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>22018.80301556858</v>
+        <v>22264.05209130449</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>22018.80301556858</v>
+        <v>22264.05209130449</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>894.8297715197593</v>
+        <v>649.5806957838544</v>
       </c>
       <c r="Q18" s="6" t="n">
         <v>0</v>
@@ -1972,13 +1972,13 @@
         <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>16024.65899843646</v>
+        <v>16203.14430508872</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>16024.65899843646</v>
+        <v>16203.14430508872</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>-16024.65899843645</v>
+        <v>-16203.14430508871</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -2037,13 +2037,13 @@
         <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>16004.59591938932</v>
+        <v>16182.85776014341</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>16004.59591938932</v>
+        <v>16182.85776014341</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>-16004.59591938448</v>
+        <v>-16182.85776013857</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -2102,13 +2102,13 @@
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>15962.25101053114</v>
+        <v>16140.04120667529</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>15962.25101053114</v>
+        <v>16140.04120667529</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-15962.25101052948</v>
+        <v>-16140.04120667363</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>0</v>
@@ -2167,13 +2167,13 @@
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>15859.08659453455</v>
+        <v>16035.72772832258</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>15859.08659453455</v>
+        <v>16035.72772832258</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>-15859.08659463373</v>
+        <v>-16035.72772842176</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2232,13 +2232,13 @@
         <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>3109.242482165629</v>
+        <v>3143.87374002514</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>2862.415452870953</v>
+        <v>2897.046710730463</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>127.8814677600924</v>
+        <v>93.25020990058148</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
@@ -2366,13 +2366,13 @@
         <v>1</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>5.221818689581455</v>
+        <v>5.279980171219437</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>5.221818689581455</v>
+        <v>5.279980171219437</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>-5.221818690141455</v>
+        <v>-5.279980171779437</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -2431,13 +2431,13 @@
         <v>1</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>1.008228251443041</v>
+        <v>1.019458064735907</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>1.008228251443041</v>
+        <v>1.019458064735907</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>1.370154972575156</v>
+        <v>1.35892515928229</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>0</v>
@@ -2496,13 +2496,13 @@
         <v>1</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>0.9098384744123992</v>
+        <v>0.9199724060689399</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>0.9098384744123992</v>
+        <v>0.9199724060689399</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>-0.9098384744123992</v>
+        <v>-0.9199724060689399</v>
       </c>
       <c r="Q27" s="6" t="n">
         <v>0</v>
@@ -2561,13 +2561,13 @@
         <v>1</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>0.3147728518743365</v>
+        <v>0.3182788440454073</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>0.3147728518743365</v>
+        <v>0.3182788440454073</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.07380726552829994</v>
+        <v>0.07030127335722904</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>0</v>
@@ -2626,13 +2626,13 @@
         <v>1</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>0.2031279690461081</v>
+        <v>0.2053904420165709</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>0.2031279690461081</v>
+        <v>0.2053904420165709</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>-0.2031279681411081</v>
+        <v>-0.2053904411115709</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -2691,13 +2691,13 @@
         <v>1</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>0.07017136754485954</v>
+        <v>0.07095294786152495</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>0.07017136754485954</v>
+        <v>0.07095294786152495</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>-0.06920133646684518</v>
+        <v>-0.06998291678351058</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>0</v>
@@ -2756,13 +2756,13 @@
         <v>1</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>0.003560864761185244</v>
+        <v>0.003600526262806552</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>0.003560864761185244</v>
+        <v>0.003600526262806552</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>0.09592513523881475</v>
+        <v>0.09588547373719344</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>0</v>
@@ -2821,13 +2821,13 @@
         <v>1</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>0.0001832417702581489</v>
+        <v>0.0001852827474520611</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0.0001832417702581489</v>
+        <v>0.0001852827474520611</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>-6.241770258148888e-06</v>
+        <v>-8.282747452061153e-06</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -2886,13 +2886,13 @@
         <v>1</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>2.017111254533797e-05</v>
+        <v>2.039578173851851e-05</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>2.017111254533797e-05</v>
+        <v>2.039578173851851e-05</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>-4.17111254533797e-06</v>
+        <v>-4.395781738518511e-06</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -2951,13 +2951,13 @@
         <v>1</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>1.838076332606629e-05</v>
+        <v>1.858549131304409e-05</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>1.838076332606629e-05</v>
+        <v>1.858549131304409e-05</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-1.436754979777128e-05</v>
+        <v>-1.457227778474909e-05</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>0</v>
@@ -3016,13 +3016,13 @@
         <v>1</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>5.390500683390287e-06</v>
+        <v>5.450540973020041e-06</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>5.390500683390287e-06</v>
+        <v>5.450540973020041e-06</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>6.094993166097132e-07</v>
+        <v>5.494590269799594e-07</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -3081,13 +3081,13 @@
         <v>1</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>3.974435608731671e-06</v>
+        <v>4.018703530967232e-06</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>3.974435608731671e-06</v>
+        <v>4.018703530967232e-06</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>-3.974435608731671e-06</v>
+        <v>-4.018703530967232e-06</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>0</v>
@@ -3146,13 +3146,13 @@
         <v>1</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>9.272277227477251e-07</v>
+        <v>9.375553387330174e-07</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>9.272277227477251e-07</v>
+        <v>9.375553387330174e-07</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>-4.378757152107251e-07</v>
+        <v>-4.482033311960174e-07</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>0</v>
@@ -3211,13 +3211,13 @@
         <v>1</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.400287909693785e-07</v>
+        <v>2.427022714076032e-07</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>2.400287909693785e-07</v>
+        <v>2.427022714076032e-07</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>-2.400287909693785e-07</v>
+        <v>-2.427022714076032e-07</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>0</v>
@@ -3276,13 +3276,13 @@
         <v>1</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>2.321288453780494e-10</v>
+        <v>2.347143349135322e-10</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>2.321288453780494e-10</v>
+        <v>2.347143349135322e-10</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>-1.08919597845378e-07</v>
+        <v>-1.089221833349135e-07</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -4678,7 +4678,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="25">
@@ -4698,7 +4698,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>7736693.016977214</v>
+        <v>7824194.465170181</v>
       </c>
     </row>
     <row r="28">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="32">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>-2942380.297009195</v>
+        <v>-2854878.848816229</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">

</xml_diff>

<commit_message>
fix(spark): S32 sUSDS POL earns DSDR, not the agent rate (sky_revenue +$888K Jan–May) (#138)
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="10">
@@ -545,7 +545,7 @@
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="n">
-        <v>7736693.016977214</v>
+        <v>7824194.465170181</v>
       </c>
     </row>
     <row r="13">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="15">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>-2942380.297009195</v>
+        <v>-2854878.848816229</v>
       </c>
     </row>
     <row r="16">
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>-7734669.938868322</v>
+        <v>-7822171.387061289</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>-1246305.303708494</v>
+        <v>-1333806.751901461</v>
       </c>
     </row>
     <row r="25">
@@ -666,7 +666,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-23T21:42:32+00:00</t>
+          <t>2026-06-25T11:40:59+00:00</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sUSDS raw / POL (ALM — Cat B 4626, demand-side spread + agent rate)</t>
+          <t>sUSDS raw / POL (ALM — Cat B 4626, demand-side spread)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -863,13 +863,13 @@
         <v>1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>1652541.117523931</v>
+        <v>1670947.3942594</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>1652541.117523931</v>
+        <v>1670947.3942594</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-518566.4581009091</v>
+        <v>-536972.7348363776</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -928,13 +928,13 @@
         <v>1</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>1534551.022002216</v>
+        <v>1551643.105506916</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>1534551.022002216</v>
+        <v>1551643.105506916</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>-1534551.022002223</v>
+        <v>-1551643.105506923</v>
       </c>
       <c r="Q3" s="6" t="n">
         <v>0</v>
@@ -993,13 +993,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>1075400.3949828</v>
+        <v>1087378.382738496</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>1075400.3949828</v>
+        <v>1087378.382738496</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>-108834.7969498004</v>
+        <v>-120812.7847054962</v>
       </c>
       <c r="Q4" s="6" t="n">
         <v>0</v>
@@ -1058,13 +1058,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>799264.5254906372</v>
+        <v>808166.8661858366</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>799264.5254906372</v>
+        <v>808166.8661858366</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>98127.554047489</v>
+        <v>89225.2133522896</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>82530624.22670487</v>
@@ -1127,13 +1127,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>608255.1096587715</v>
+        <v>615029.9558368304</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>608255.1096587715</v>
+        <v>615029.9558368304</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>242650.3515826334</v>
+        <v>235875.5054045745</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>0</v>
@@ -1192,13 +1192,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>458119.2897228166</v>
+        <v>463221.8982661542</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>458119.2897228166</v>
+        <v>463221.8982661542</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-219429.4613868165</v>
+        <v>-224532.0699301542</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>0</v>
@@ -1257,13 +1257,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>320482.1759169488</v>
+        <v>324051.7594850424</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>320482.1759169488</v>
+        <v>324051.7594850424</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-313050.5173337357</v>
+        <v>-316620.1009018293</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>0</v>
@@ -1322,13 +1322,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>302720.865516389</v>
+        <v>306092.6206668108</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>302720.865516389</v>
+        <v>306092.6206668108</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>155557.645037369</v>
+        <v>152185.8898869471</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>95188953.04035926</v>
@@ -1391,13 +1391,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>263763.8552620765</v>
+        <v>266701.7007784666</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>242824.9773189502</v>
+        <v>245762.8228353402</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>-10487.79839418177</v>
+        <v>-13425.6439105718</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
@@ -1456,13 +1456,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>239815.1255672291</v>
+        <v>242486.2261648078</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>220777.4161048071</v>
+        <v>223448.5167023858</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>9863.46688124739</v>
+        <v>7192.366283668689</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -1521,13 +1521,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>155985.0667378869</v>
+        <v>157722.4542525044</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>155985.0667378869</v>
+        <v>157722.4542525044</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>62136.39805438424</v>
+        <v>60399.01053976677</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>0</v>
@@ -1586,13 +1586,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>138410.399456311</v>
+        <v>139952.0374152363</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>138410.399456311</v>
+        <v>139952.0374152363</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>7082.032676688972</v>
+        <v>5540.394717763749</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -1651,13 +1651,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>137510.7557385326</v>
+        <v>139042.3733166896</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>126594.4725828467</v>
+        <v>128126.0901610037</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>-5239.892153737481</v>
+        <v>-6771.509731894468</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
@@ -1777,13 +1777,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>48149.2551643835</v>
+        <v>48685.54954505841</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>48149.2551643835</v>
+        <v>48685.54954505841</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>34465.38674161991</v>
+        <v>33929.09236094499</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>0</v>
@@ -1842,13 +1842,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>32046.35286660667</v>
+        <v>32403.29045379908</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>32046.35286660667</v>
+        <v>32403.29045379908</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>-449.4019886066722</v>
+        <v>-806.3395757990797</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>0</v>
@@ -1907,13 +1907,13 @@
         <v>1</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>22018.80301556858</v>
+        <v>22264.05209130449</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>22018.80301556858</v>
+        <v>22264.05209130449</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>894.8297715197593</v>
+        <v>649.5806957838544</v>
       </c>
       <c r="Q18" s="6" t="n">
         <v>0</v>
@@ -1972,13 +1972,13 @@
         <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>16024.65899843646</v>
+        <v>16203.14430508872</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>16024.65899843646</v>
+        <v>16203.14430508872</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>-16024.65899843645</v>
+        <v>-16203.14430508871</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -2037,13 +2037,13 @@
         <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>16004.59591938932</v>
+        <v>16182.85776014341</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>16004.59591938932</v>
+        <v>16182.85776014341</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>-16004.59591938448</v>
+        <v>-16182.85776013857</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -2102,13 +2102,13 @@
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>15962.25101053114</v>
+        <v>16140.04120667529</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>15962.25101053114</v>
+        <v>16140.04120667529</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-15962.25101052948</v>
+        <v>-16140.04120667363</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>0</v>
@@ -2167,13 +2167,13 @@
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>15859.08659453455</v>
+        <v>16035.72772832258</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>15859.08659453455</v>
+        <v>16035.72772832258</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>-15859.08659463373</v>
+        <v>-16035.72772842176</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2232,13 +2232,13 @@
         <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>3109.242482165629</v>
+        <v>3143.87374002514</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>2862.415452870953</v>
+        <v>2897.046710730463</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>127.8814677600924</v>
+        <v>93.25020990058148</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
@@ -2366,13 +2366,13 @@
         <v>1</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>5.221818689581455</v>
+        <v>5.279980171219437</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>5.221818689581455</v>
+        <v>5.279980171219437</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>-5.221818690141455</v>
+        <v>-5.279980171779437</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -2431,13 +2431,13 @@
         <v>1</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>1.008228251443041</v>
+        <v>1.019458064735907</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>1.008228251443041</v>
+        <v>1.019458064735907</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>1.370154972575156</v>
+        <v>1.35892515928229</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>0</v>
@@ -2496,13 +2496,13 @@
         <v>1</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>0.9098384744123992</v>
+        <v>0.9199724060689399</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>0.9098384744123992</v>
+        <v>0.9199724060689399</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>-0.9098384744123992</v>
+        <v>-0.9199724060689399</v>
       </c>
       <c r="Q27" s="6" t="n">
         <v>0</v>
@@ -2561,13 +2561,13 @@
         <v>1</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>0.3147728518743365</v>
+        <v>0.3182788440454073</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>0.3147728518743365</v>
+        <v>0.3182788440454073</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.07380726552829994</v>
+        <v>0.07030127335722904</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>0</v>
@@ -2626,13 +2626,13 @@
         <v>1</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>0.2031279690461081</v>
+        <v>0.2053904420165709</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>0.2031279690461081</v>
+        <v>0.2053904420165709</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>-0.2031279681411081</v>
+        <v>-0.2053904411115709</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -2691,13 +2691,13 @@
         <v>1</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>0.07017136754485954</v>
+        <v>0.07095294786152495</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>0.07017136754485954</v>
+        <v>0.07095294786152495</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>-0.06920133646684518</v>
+        <v>-0.06998291678351058</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>0</v>
@@ -2756,13 +2756,13 @@
         <v>1</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>0.003560864761185244</v>
+        <v>0.003600526262806552</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>0.003560864761185244</v>
+        <v>0.003600526262806552</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>0.09592513523881475</v>
+        <v>0.09588547373719344</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>0</v>
@@ -2821,13 +2821,13 @@
         <v>1</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>0.0001832417702581489</v>
+        <v>0.0001852827474520611</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0.0001832417702581489</v>
+        <v>0.0001852827474520611</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>-6.241770258148888e-06</v>
+        <v>-8.282747452061153e-06</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -2886,13 +2886,13 @@
         <v>1</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>2.017111254533797e-05</v>
+        <v>2.039578173851851e-05</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>2.017111254533797e-05</v>
+        <v>2.039578173851851e-05</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>-4.17111254533797e-06</v>
+        <v>-4.395781738518511e-06</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -2951,13 +2951,13 @@
         <v>1</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>1.838076332606629e-05</v>
+        <v>1.858549131304409e-05</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>1.838076332606629e-05</v>
+        <v>1.858549131304409e-05</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-1.436754979777128e-05</v>
+        <v>-1.457227778474909e-05</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>0</v>
@@ -3016,13 +3016,13 @@
         <v>1</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>5.390500683390287e-06</v>
+        <v>5.450540973020041e-06</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>5.390500683390287e-06</v>
+        <v>5.450540973020041e-06</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>6.094993166097132e-07</v>
+        <v>5.494590269799594e-07</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -3081,13 +3081,13 @@
         <v>1</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>3.974435608731671e-06</v>
+        <v>4.018703530967232e-06</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>3.974435608731671e-06</v>
+        <v>4.018703530967232e-06</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>-3.974435608731671e-06</v>
+        <v>-4.018703530967232e-06</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>0</v>
@@ -3146,13 +3146,13 @@
         <v>1</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>9.272277227477251e-07</v>
+        <v>9.375553387330174e-07</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>9.272277227477251e-07</v>
+        <v>9.375553387330174e-07</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>-4.378757152107251e-07</v>
+        <v>-4.482033311960174e-07</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>0</v>
@@ -3211,13 +3211,13 @@
         <v>1</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.400287909693785e-07</v>
+        <v>2.427022714076032e-07</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>2.400287909693785e-07</v>
+        <v>2.427022714076032e-07</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>-2.400287909693785e-07</v>
+        <v>-2.427022714076032e-07</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>0</v>
@@ -3276,13 +3276,13 @@
         <v>1</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>2.321288453780494e-10</v>
+        <v>2.347143349135322e-10</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>2.321288453780494e-10</v>
+        <v>2.347143349135322e-10</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>-1.08919597845378e-07</v>
+        <v>-1.089221833349135e-07</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -4678,7 +4678,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="25">
@@ -4698,7 +4698,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>7736693.016977214</v>
+        <v>7824194.465170181</v>
       </c>
     </row>
     <row r="28">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>7734669.938868322</v>
+        <v>7822171.387061289</v>
       </c>
     </row>
     <row r="32">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>-2942380.297009195</v>
+        <v>-2854878.848816229</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">

</xml_diff>

<commit_message>
chore(dr): bump settle-dr-dune to d9c469a + refresh Spark DR (+4 ref codes)
Update the settle-dr-dune submodule a8d3aee → d9c469a (their PR #5) and
refresh Distribution Rewards via `--dr-only` (no recompute — no RPC/Dune).

Only Spark changed: the new workbook adds 4 ref codes (30 → 34) and nudges
per-month DR up by ~$8–16K (Jan 1,144,088 → 1,154,488 … May 1,622,763 →
1,632,541); prime_agent_total_revenue / prime profit rise by the same,
sky_revenue unchanged. Grove / Skybase / Keel DR are unchanged in this
workbook revision (no report change).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -511,13 +511,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1144088.13</v>
+        <v>1154488.13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>8753785.242841383</v>
+        <v>8764185.242841383</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
chore(dr): bump settle-dr-dune to d9c469a + refresh Spark DR (+4 ref codes) (#140)
Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -511,13 +511,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1144088.13</v>
+        <v>1154488.13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>8753785.242841383</v>
+        <v>8764185.242841383</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
feat(spark): source Uni v4 flows from Dune + v4-aware Jan–Jun reports
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-03T07:16:58+00:00</t>
+          <t>2026-07-07T00:00:41+00:00</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S62"/>
+  <dimension ref="A1:S64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3699,12 +3699,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S26</t>
+          <t>S61</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>USDC raw (ALM idle)</t>
+          <t>Spark.fi PYUSD Reserve Uniswap V4 (PYUSD/USDS)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
@@ -3727,13 +3727,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>891780.0000000449</v>
+        <v>0</v>
       </c>
       <c r="I46" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J46" s="6" t="n">
-        <v>891780.0000000449</v>
+        <v>0</v>
       </c>
       <c r="K46" s="6" t="n">
         <v>0</v>
@@ -3751,7 +3751,7 @@
         <v>0</v>
       </c>
       <c r="P46" s="6" t="n">
-        <v>891780.0000000449</v>
+        <v>0</v>
       </c>
       <c r="Q46" s="6" t="n">
         <v>0</v>
@@ -3764,12 +3764,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>S29</t>
+          <t>S62</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>DAI raw (ALM idle)</t>
+          <t>Spark.fi USDT Reserve Uniswap V4 (USDT/USDS)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
@@ -3792,13 +3792,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>1.4391531e-08</v>
+        <v>0</v>
       </c>
       <c r="I47" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>1.4391531e-08</v>
+        <v>0</v>
       </c>
       <c r="K47" s="6" t="n">
         <v>0</v>
@@ -3816,7 +3816,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="6" t="n">
-        <v>1.4391531e-08</v>
+        <v>0</v>
       </c>
       <c r="Q47" s="6" t="n">
         <v>0</v>
@@ -3829,12 +3829,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S31</t>
+          <t>S26</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
+          <t>USDC raw (ALM idle)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3857,22 +3857,22 @@
         <v>0</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>-7.90813362735e-08</v>
+        <v>891780.0000000449</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J48" s="6" t="n">
-        <v>-7.90813362735e-08</v>
+        <v>891780.0000000449</v>
       </c>
       <c r="K48" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L48" s="6" t="n">
-        <v>1.422012653983871e-08</v>
+        <v>0</v>
       </c>
       <c r="M48" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N48" s="6" t="n">
         <v>0</v>
@@ -3881,7 +3881,7 @@
         <v>0</v>
       </c>
       <c r="P48" s="6" t="n">
-        <v>-7.90813362735e-08</v>
+        <v>891780.0000000449</v>
       </c>
       <c r="Q48" s="6" t="n">
         <v>0</v>
@@ -3889,26 +3889,22 @@
       <c r="R48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t>CoF excluded (Savings V2 depositor capital; not in cum_alm_usds)</t>
-        </is>
-      </c>
+      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S38</t>
+          <t>S29</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>USDS raw (Base — POL)</t>
+          <t>DAI raw (ALM idle)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3917,31 +3913,31 @@
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0</v>
+        <v>1.4391531e-08</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J49" s="6" t="n">
-        <v>0</v>
+        <v>1.4391531e-08</v>
       </c>
       <c r="K49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="M49" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N49" s="6" t="n">
         <v>0</v>
@@ -3950,39 +3946,35 @@
         <v>0</v>
       </c>
       <c r="P49" s="6" t="n">
-        <v>0</v>
+        <v>1.4391531e-08</v>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="R49" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S42</t>
+          <t>S31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
+          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
@@ -3995,22 +3987,22 @@
         <v>0</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0</v>
+        <v>-7.90813362735e-08</v>
       </c>
       <c r="I50" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J50" s="6" t="n">
-        <v>0</v>
+        <v>-7.90813362735e-08</v>
       </c>
       <c r="K50" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L50" s="6" t="n">
-        <v>0</v>
+        <v>1.422012653983871e-08</v>
       </c>
       <c r="M50" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N50" s="6" t="n">
         <v>0</v>
@@ -4019,7 +4011,7 @@
         <v>0</v>
       </c>
       <c r="P50" s="6" t="n">
-        <v>0</v>
+        <v>-7.90813362735e-08</v>
       </c>
       <c r="Q50" s="6" t="n">
         <v>0</v>
@@ -4027,22 +4019,26 @@
       <c r="R50" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>CoF excluded (Savings V2 depositor capital; not in cum_alm_usds)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S44</t>
+          <t>S38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>USDS raw (Arbitrum — POL)</t>
+          <t>USDS raw (Base — POL)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4051,10 +4047,10 @@
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>
@@ -4072,7 +4068,7 @@
         <v>0</v>
       </c>
       <c r="L51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="M51" s="7" t="n">
         <v>0</v>
@@ -4087,7 +4083,7 @@
         <v>0</v>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="R51" s="6" t="n">
         <v>0</v>
@@ -4101,29 +4097,29 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S48</t>
+          <t>S42</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>USDS raw (Optimism — POL)</t>
+          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="F52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="G52" s="6" t="n">
         <v>0</v>
@@ -4141,10 +4137,10 @@
         <v>0</v>
       </c>
       <c r="L52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="M52" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N52" s="6" t="n">
         <v>0</v>
@@ -4156,31 +4152,27 @@
         <v>0</v>
       </c>
       <c r="Q52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="R52" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S52</t>
+          <t>S44</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>USDS raw (Unichain — POL)</t>
+          <t>USDS raw (Arbitrum — POL)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4189,10 +4181,10 @@
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="G53" s="6" t="n">
         <v>0</v>
@@ -4210,7 +4202,7 @@
         <v>0</v>
       </c>
       <c r="L53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="M53" s="7" t="n">
         <v>0</v>
@@ -4225,7 +4217,7 @@
         <v>0</v>
       </c>
       <c r="Q53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="R53" s="6" t="n">
         <v>0</v>
@@ -4239,168 +4231,250 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>S48</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>USDS raw (Optimism — POL)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>optimism</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="M54" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="R54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>S52</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>USDS raw (Unichain — POL)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>unichain</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="M55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="R55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S54" t="inlineStr">
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S56" t="inlineStr">
         <is>
           <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Position-only venues (PnL aggregated at prime level)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Pricing cat.</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>Position SoM</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Position EoM</t>
         </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>S56</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spUSDC vault</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="n">
-        <v>215278739.036717</v>
-      </c>
-      <c r="F58" s="6" t="n">
-        <v>207131500.431691</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>S57</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spUSDT vault</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="n">
-        <v>153856441.430568</v>
-      </c>
-      <c r="F59" s="6" t="n">
-        <v>120038508.359851</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S59</t>
+          <t>S56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Spark Savings V2 — spPYUSD vault</t>
+          <t>Spark Savings V2 — spUSDC vault</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -4414,51 +4488,107 @@
         </is>
       </c>
       <c r="E60" s="6" t="n">
-        <v>21463.341472</v>
+        <v>215278739.036717</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>285387.136685</v>
+        <v>207131500.431691</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>S57</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spUSDT vault</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>153856441.430568</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>120038508.359851</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>S59</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spPYUSD vault</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>21463.341472</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>285387.136685</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>S60</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Spark Savings V2 — spUSDC vault (Avalanche-C, CREATE2 same address)</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>avalanche_c</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="E61" s="6" t="n">
+      <c r="E63" s="6" t="n">
         <v>190414182.348414</v>
       </c>
-      <c r="F61" s="6" t="n">
+      <c r="F63" s="6" t="n">
         <v>95656876.179346</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" s="5" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>Aggregated actual_revenue (included in prime_agent_revenue, not in Venues body above)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" s="9" t="n">
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4875,7 +5005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5035,6 +5165,86 @@
       </c>
       <c r="J5" s="6" t="n">
         <v>2023.078108892489</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S61</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PYUSD in PYUSD/USDS Uniswap V4</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>S62</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>USDT in USDT/USDS Uniswap V4</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(june): June 2026 settlements for all primes (+fixture refresh through 06-30) (#144)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
+++ b/settlements/spark/2026-01/spark_settlement_january_2026.xlsx
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7503304.563025013</v>
+        <v>7503304.563024798</v>
       </c>
     </row>
     <row r="5">
@@ -517,7 +517,7 @@
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>8764185.242841383</v>
+        <v>8764185.242841169</v>
       </c>
     </row>
     <row r="9">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>7503304.563025013</v>
+        <v>7503304.563024798</v>
       </c>
     </row>
     <row r="23">
@@ -641,7 +641,7 @@
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" s="4" t="n">
-        <v>-1333806.751901461</v>
+        <v>-1333806.751901675</v>
       </c>
     </row>
     <row r="26">
@@ -676,7 +676,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-06-25T22:30:37+00:00</t>
+          <t>2026-07-07T00:00:41+00:00</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S62"/>
+  <dimension ref="A1:S64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -855,13 +855,13 @@
         <v>-136047042.8806877</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>1133974.659423022</v>
+        <v>1133974.659423013</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>1133974.659423022</v>
+        <v>1133974.659423013</v>
       </c>
       <c r="K2" s="6" t="n">
         <v>0</v>
@@ -879,7 +879,7 @@
         <v>1670947.3942594</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-536972.7348363776</v>
+        <v>-536972.7348363873</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -920,13 +920,13 @@
         <v>46123644.716281</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>-7.512e-09</v>
+        <v>-4.089e-09</v>
       </c>
       <c r="I3" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>-7.512e-09</v>
+        <v>-4.089e-09</v>
       </c>
       <c r="K3" s="6" t="n">
         <v>0</v>
@@ -944,7 +944,7 @@
         <v>1551643.105506916</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>-1551643.105506923</v>
+        <v>-1551643.10550692</v>
       </c>
       <c r="Q3" s="6" t="n">
         <v>0</v>
@@ -1074,7 +1074,7 @@
         <v>808166.8661858366</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>89225.2133522896</v>
+        <v>89225.21335228962</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>82530624.22670487</v>
@@ -1119,13 +1119,13 @@
         <v>-200000439.4950232</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>850905.4612414049</v>
+        <v>850905.4612414278</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>850905.4612414049</v>
+        <v>850905.4612414278</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>0</v>
@@ -1137,13 +1137,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>615029.9558368304</v>
+        <v>615029.9558368303</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>615029.9558368304</v>
+        <v>615029.9558368303</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>235875.5054045745</v>
+        <v>235875.5054045975</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>0</v>
@@ -1407,7 +1407,7 @@
         <v>245762.8228353402</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>-13425.6439105718</v>
+        <v>-13425.64391057179</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
@@ -1466,13 +1466,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>242486.2261648078</v>
+        <v>242486.2261648077</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>223448.5167023858</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7192.366283668689</v>
+        <v>7192.366283668691</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -1513,31 +1513,31 @@
         <v>-167771790.9797579</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>218121.4647922712</v>
+        <v>218121.4647920985</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>218121.4647922712</v>
+        <v>218121.4647920985</v>
       </c>
       <c r="K12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>48672080.32484906</v>
+        <v>48672080.32484919</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>157722.4542525044</v>
+        <v>157722.4542525048</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>157722.4542525044</v>
+        <v>157722.4542525048</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>60399.01053976677</v>
+        <v>60399.01053959369</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>0</v>
@@ -1602,7 +1602,7 @@
         <v>139952.0374152363</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5540.394717763749</v>
+        <v>5540.394717763751</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -1667,7 +1667,7 @@
         <v>128126.0901610037</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>-6771.509731894468</v>
+        <v>-6771.509731894467</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
@@ -1793,7 +1793,7 @@
         <v>48685.54954505841</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>33929.09236094499</v>
+        <v>33929.092360945</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>0</v>
@@ -1858,7 +1858,7 @@
         <v>32403.29045379908</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>-806.3395757990797</v>
+        <v>-806.3395757990795</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>0</v>
@@ -1923,7 +1923,7 @@
         <v>22264.05209130449</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>649.5806957838544</v>
+        <v>649.5806957838545</v>
       </c>
       <c r="Q18" s="6" t="n">
         <v>0</v>
@@ -1964,13 +1964,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>8e-12</v>
+        <v>4.68e-11</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>8e-12</v>
+        <v>4.68e-11</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>0</v>
@@ -1988,7 +1988,7 @@
         <v>16203.14430508872</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>-16203.14430508871</v>
+        <v>-16203.14430508868</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -2029,31 +2029,31 @@
         <v>-5182.684447</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>4.83813e-09</v>
+        <v>1.002278e-08</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>4.83813e-09</v>
+        <v>1.002278e-08</v>
       </c>
       <c r="K20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>4993920.215864256</v>
+        <v>4993920.215864252</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>16182.85776014341</v>
+        <v>16182.8577601434</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>16182.85776014341</v>
+        <v>16182.8577601434</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>-16182.85776013857</v>
+        <v>-16182.85776013337</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -2094,19 +2094,19 @@
         <v>0</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1.658e-09</v>
+        <v>1.053e-09</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1.658e-09</v>
+        <v>1.053e-09</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>4980707.317678578</v>
+        <v>4980707.317678579</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>1</v>
@@ -2118,7 +2118,7 @@
         <v>16140.04120667529</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-16140.04120667363</v>
+        <v>-16140.04120667424</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>0</v>
@@ -2159,31 +2159,31 @@
         <v>247035.172535</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>-9.9179e-08</v>
+        <v>-8.469500000000001e-08</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>-9.9179e-08</v>
+        <v>-8.469500000000001e-08</v>
       </c>
       <c r="K22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>4948516.885305397</v>
+        <v>4948516.885305393</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>16035.72772832258</v>
+        <v>16035.72772832256</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>16035.72772832258</v>
+        <v>16035.72772832256</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>-16035.72772842176</v>
+        <v>-16035.72772840726</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2248,7 +2248,7 @@
         <v>2897.046710730463</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>93.25020990058148</v>
+        <v>93.25020990058151</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
@@ -2358,31 +2358,31 @@
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>-5.6e-10</v>
+        <v>-2.95e-09</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>-5.6e-10</v>
+        <v>-2.95e-09</v>
       </c>
       <c r="K25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>1629.366092641322</v>
+        <v>1629.366092642247</v>
       </c>
       <c r="M25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>5.279980171219437</v>
+        <v>5.279980171222434</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>5.279980171219437</v>
+        <v>5.279980171222434</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>-5.279980171779437</v>
+        <v>-5.279980174172434</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -2618,31 +2618,31 @@
         <v>0</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>9.05e-10</v>
+        <v>4.4347e-08</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>9.05e-10</v>
+        <v>4.4347e-08</v>
       </c>
       <c r="K29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>63.38209825078258</v>
+        <v>63.38209822987316</v>
       </c>
       <c r="M29" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>0.2053904420165709</v>
+        <v>0.2053904419488137</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>0.2053904420165709</v>
+        <v>0.2053904419488137</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>-0.2053904411115709</v>
+        <v>-0.2053903976018137</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -2837,7 +2837,7 @@
         <v>0.0001852827474520611</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>-8.282747452061153e-06</v>
+        <v>-8.282747452061152e-06</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -2902,7 +2902,7 @@
         <v>2.039578173851851e-05</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>-4.395781738518511e-06</v>
+        <v>-4.39578173851851e-06</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -3032,7 +3032,7 @@
         <v>5.450540973020041e-06</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>5.494590269799594e-07</v>
+        <v>5.494590269799595e-07</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -3091,13 +3091,13 @@
         <v>1</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>4.018703530967232e-06</v>
+        <v>4.018703530967231e-06</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>4.018703530967232e-06</v>
+        <v>4.018703530967231e-06</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>-4.018703530967232e-06</v>
+        <v>-4.018703530967231e-06</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>0</v>
@@ -3240,12 +3240,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S29</t>
+          <t>S9</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DAI raw (ALM idle)</t>
+          <t>Aave Ethereum USDT (aToken)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
@@ -3268,31 +3268,31 @@
         <v>0</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>-1.08687469e-07</v>
+        <v>0</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>-1.08687469e-07</v>
+        <v>0</v>
       </c>
       <c r="K39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>7.243125283870968e-08</v>
+        <v>0</v>
       </c>
       <c r="M39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>2.347143349135322e-10</v>
+        <v>0</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>2.347143349135322e-10</v>
+        <v>0</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>-1.089221833349135e-07</v>
+        <v>0</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -3305,12 +3305,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Aave Ethereum USDT (aToken)</t>
+          <t>Spark Blue Chip USDT Vault (Morpho V2)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
@@ -3370,12 +3370,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Spark Blue Chip USDT Vault (Morpho V2)</t>
+          <t>Maple syrupUSDT (ERC-4626)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3435,12 +3435,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S15</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Maple syrupUSDT (ERC-4626)</t>
+          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
@@ -3500,12 +3500,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S19</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
+          <t>Janus Henderson Anemoy Treasury Fund (JTRSY)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3565,12 +3565,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S20</t>
+          <t>S21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Janus Henderson Anemoy Treasury Fund (JTRSY)</t>
+          <t>Superstate Short Duration US Government Securities Fund (USTB)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3608,7 +3608,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N44" s="6" t="n">
         <v>0</v>
@@ -3625,17 +3625,21 @@
       <c r="R44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>SDE (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S21</t>
+          <t>S22</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Superstate Short Duration US Government Securities Fund (USTB)</t>
+          <t>Superstate Crypto Carry Fund (USCC)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3673,7 +3677,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N45" s="6" t="n">
         <v>0</v>
@@ -3690,21 +3694,17 @@
       <c r="R45" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>SDE (fixed)</t>
-        </is>
-      </c>
+      <c r="S45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S22</t>
+          <t>S61</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Superstate Crypto Carry Fund (USCC)</t>
+          <t>Spark.fi PYUSD Reserve Uniswap V4 (PYUSD/USDS)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
@@ -3764,12 +3764,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>S26</t>
+          <t>S62</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>USDC raw (ALM idle)</t>
+          <t>Spark.fi USDT Reserve Uniswap V4 (USDT/USDS)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
@@ -3792,13 +3792,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>891780.0000001139</v>
+        <v>0</v>
       </c>
       <c r="I47" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>891780.0000001139</v>
+        <v>0</v>
       </c>
       <c r="K47" s="6" t="n">
         <v>0</v>
@@ -3816,7 +3816,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="6" t="n">
-        <v>891780.0000001139</v>
+        <v>0</v>
       </c>
       <c r="Q47" s="6" t="n">
         <v>0</v>
@@ -3829,12 +3829,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S31</t>
+          <t>S26</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
+          <t>USDC raw (ALM idle)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3857,13 +3857,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>9.31926637265e-08</v>
+        <v>891780.0000000449</v>
       </c>
       <c r="I48" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J48" s="6" t="n">
-        <v>9.31926637265e-08</v>
+        <v>891780.0000000449</v>
       </c>
       <c r="K48" s="6" t="n">
         <v>0</v>
@@ -3872,7 +3872,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N48" s="6" t="n">
         <v>0</v>
@@ -3881,7 +3881,7 @@
         <v>0</v>
       </c>
       <c r="P48" s="6" t="n">
-        <v>9.31926637265e-08</v>
+        <v>891780.0000000449</v>
       </c>
       <c r="Q48" s="6" t="n">
         <v>0</v>
@@ -3889,26 +3889,22 @@
       <c r="R48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S38</t>
+          <t>S29</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>USDS raw (Base — POL)</t>
+          <t>DAI raw (ALM idle)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3917,31 +3913,31 @@
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0</v>
+        <v>1.4391531e-08</v>
       </c>
       <c r="I49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J49" s="6" t="n">
-        <v>0</v>
+        <v>1.4391531e-08</v>
       </c>
       <c r="K49" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="M49" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N49" s="6" t="n">
         <v>0</v>
@@ -3950,39 +3946,35 @@
         <v>0</v>
       </c>
       <c r="P49" s="6" t="n">
-        <v>0</v>
+        <v>1.4391531e-08</v>
       </c>
       <c r="Q49" s="6" t="n">
-        <v>65170000</v>
+        <v>0</v>
       </c>
       <c r="R49" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S42</t>
+          <t>S31</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
+          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
@@ -3995,22 +3987,22 @@
         <v>0</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0</v>
+        <v>-7.90813362735e-08</v>
       </c>
       <c r="I50" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J50" s="6" t="n">
-        <v>0</v>
+        <v>-7.90813362735e-08</v>
       </c>
       <c r="K50" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L50" s="6" t="n">
-        <v>0</v>
+        <v>1.422012653983871e-08</v>
       </c>
       <c r="M50" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N50" s="6" t="n">
         <v>0</v>
@@ -4019,7 +4011,7 @@
         <v>0</v>
       </c>
       <c r="P50" s="6" t="n">
-        <v>0</v>
+        <v>-7.90813362735e-08</v>
       </c>
       <c r="Q50" s="6" t="n">
         <v>0</v>
@@ -4027,22 +4019,26 @@
       <c r="R50" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>CoF excluded (Savings V2 depositor capital; not in cum_alm_usds)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S44</t>
+          <t>S38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>USDS raw (Arbitrum — POL)</t>
+          <t>USDS raw (Base — POL)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4051,10 +4047,10 @@
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>
@@ -4072,7 +4068,7 @@
         <v>0</v>
       </c>
       <c r="L51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="M51" s="7" t="n">
         <v>0</v>
@@ -4087,7 +4083,7 @@
         <v>0</v>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>90000000</v>
+        <v>65170000</v>
       </c>
       <c r="R51" s="6" t="n">
         <v>0</v>
@@ -4101,29 +4097,29 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S48</t>
+          <t>S42</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>USDS raw (Optimism — POL)</t>
+          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="F52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="G52" s="6" t="n">
         <v>0</v>
@@ -4141,10 +4137,10 @@
         <v>0</v>
       </c>
       <c r="L52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="M52" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N52" s="6" t="n">
         <v>0</v>
@@ -4156,31 +4152,27 @@
         <v>0</v>
       </c>
       <c r="Q52" s="6" t="n">
-        <v>89900000</v>
+        <v>0</v>
       </c>
       <c r="R52" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S52</t>
+          <t>S44</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>USDS raw (Unichain — POL)</t>
+          <t>USDS raw (Arbitrum — POL)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4189,10 +4181,10 @@
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="G53" s="6" t="n">
         <v>0</v>
@@ -4210,7 +4202,7 @@
         <v>0</v>
       </c>
       <c r="L53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="M53" s="7" t="n">
         <v>0</v>
@@ -4225,7 +4217,7 @@
         <v>0</v>
       </c>
       <c r="Q53" s="6" t="n">
-        <v>89900000</v>
+        <v>90000000</v>
       </c>
       <c r="R53" s="6" t="n">
         <v>0</v>
@@ -4239,168 +4231,250 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>S48</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>USDS raw (Optimism — POL)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>optimism</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="M54" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="R54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>S52</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>USDS raw (Unichain — POL)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>unichain</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="M55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="6" t="n">
+        <v>89900000</v>
+      </c>
+      <c r="R55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S54" t="inlineStr">
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S56" t="inlineStr">
         <is>
           <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Position-only venues (PnL aggregated at prime level)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Pricing cat.</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>Position SoM</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Position EoM</t>
         </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>S56</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spUSDC vault</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="n">
-        <v>215278739.036717</v>
-      </c>
-      <c r="F58" s="6" t="n">
-        <v>207131500.431691</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>S57</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spUSDT vault</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="n">
-        <v>153856441.430568</v>
-      </c>
-      <c r="F59" s="6" t="n">
-        <v>120038508.359851</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S59</t>
+          <t>S56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Spark Savings V2 — spPYUSD vault</t>
+          <t>Spark Savings V2 — spUSDC vault</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -4414,51 +4488,107 @@
         </is>
       </c>
       <c r="E60" s="6" t="n">
-        <v>21463.341472</v>
+        <v>215278739.036717</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>285387.136685</v>
+        <v>207131500.431691</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>S57</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spUSDT vault</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>153856441.430568</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>120038508.359851</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>S59</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spPYUSD vault</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>21463.341472</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>285387.136685</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>S60</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Spark Savings V2 — spUSDC vault (Avalanche-C, CREATE2 same address)</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>avalanche_c</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="E61" s="6" t="n">
+      <c r="E63" s="6" t="n">
         <v>190414182.348414</v>
       </c>
-      <c r="F61" s="6" t="n">
+      <c r="F63" s="6" t="n">
         <v>95656876.179346</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" s="5" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>Aggregated actual_revenue (included in prime_agent_revenue, not in Venues body above)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" s="9" t="n">
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4875,7 +5005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5035,6 +5165,86 @@
       </c>
       <c r="J5" s="6" t="n">
         <v>2023.078108892489</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S61</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PYUSD in PYUSD/USDS Uniswap V4</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>S62</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>USDT in USDT/USDS Uniswap V4</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>